<commit_message>
Add gym accessories and expand rehab equipment
</commit_message>
<xml_diff>
--- a/outputs/wyposazenie-silowni/wyposazenie-silowni-zsz5-2027.xlsx
+++ b/outputs/wyposazenie-silowni/wyposazenie-silowni-zsz5-2027.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Podsumowanie" sheetId="1" r:id="R171e7bb4994c42b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kosztorys siłowni" sheetId="2" r:id="R39eac3f7aaa54c2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Podsumowanie" sheetId="1" r:id="Rf3b5b6b067744a7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kosztorys siłowni" sheetId="2" r:id="Ra973be4e75454619"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -348,7 +348,7 @@
         <x:v>Liczba pozycji</x:v>
       </x:c>
       <x:c r="B4" s="6" t="n">
-        <x:v>17</x:v>
+        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -364,8 +364,8 @@
         <x:v>Suma cen sprzętu</x:v>
       </x:c>
       <x:c r="B6" s="10" t="n">
-        <x:f>'Kosztorys siłowni'!F20</x:f>
-        <x:v>117063.59</x:v>
+        <x:f>'Kosztorys siłowni'!F29</x:f>
+        <x:v>154627.97999999995</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -373,8 +373,8 @@
         <x:v>Prognozowana suma +20%</x:v>
       </x:c>
       <x:c r="B7" s="12" t="n">
-        <x:f>'Kosztorys siłowni'!G20</x:f>
-        <x:v>140476.308</x:v>
+        <x:f>'Kosztorys siłowni'!G29</x:f>
+        <x:v>185553.57599999994</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -405,16 +405,16 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$18,'Kosztorys siłowni'!$A$2:$A$18,A11)</x:f>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$27,'Kosztorys siłowni'!$A$2:$A$27,A11)</x:f>
         <x:v>16297</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$18,'Kosztorys siłowni'!$A$2:$A$18,A11)</x:f>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$27,'Kosztorys siłowni'!$A$2:$A$27,A11)</x:f>
         <x:v>19556.399999999998</x:v>
       </x:c>
       <x:c r="E11" s="15" t="n">
         <x:f>D11/$B$7</x:f>
-        <x:v>0.1392149343788278</x:v>
+        <x:v>0.105394896835618</x:v>
       </x:c>
       <x:c r="F11" s="6" t="str"/>
     </x:row>
@@ -423,147 +423,210 @@
         <x:v>Wolne ciężary</x:v>
       </x:c>
       <x:c r="B12" s="6" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C12" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$18,'Kosztorys siłowni'!$A$2:$A$18,A12)</x:f>
-        <x:v>11622.61</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$27,'Kosztorys siłowni'!$A$2:$A$27,A12)</x:f>
+        <x:v>12372.6</x:v>
       </x:c>
       <x:c r="D12" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$18,'Kosztorys siłowni'!$A$2:$A$18,A12)</x:f>
-        <x:v>13947.132</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$27,'Kosztorys siłowni'!$A$2:$A$27,A12)</x:f>
+        <x:v>14847.119999999999</x:v>
       </x:c>
       <x:c r="E12" s="15" t="n">
         <x:f>D12/$B$7</x:f>
-        <x:v>0.09928458541208245</x:v>
+        <x:v>0.08001527278568861</x:v>
       </x:c>
       <x:c r="F12" s="6" t="str"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="6" t="str">
-        <x:v>Maszyny siłowe</x:v>
+        <x:v>Przechowywanie</x:v>
       </x:c>
       <x:c r="B13" s="6" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C13" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$18,'Kosztorys siłowni'!$A$2:$A$18,A13)</x:f>
-        <x:v>15190.38</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$27,'Kosztorys siłowni'!$A$2:$A$27,A13)</x:f>
+        <x:v>921.31</x:v>
       </x:c>
       <x:c r="D13" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$18,'Kosztorys siłowni'!$A$2:$A$18,A13)</x:f>
-        <x:v>18228.456</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$27,'Kosztorys siłowni'!$A$2:$A$27,A13)</x:f>
+        <x:v>1105.572</x:v>
       </x:c>
       <x:c r="E13" s="15" t="n">
         <x:f>D13/$B$7</x:f>
-        <x:v>0.12976178160946542</x:v>
+        <x:v>0.005958236019121509</x:v>
       </x:c>
       <x:c r="F13" s="6" t="str"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="6" t="str">
-        <x:v>Maszyny na nogi</x:v>
+        <x:v>Maszyny siłowe</x:v>
       </x:c>
       <x:c r="B14" s="6" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C14" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$18,'Kosztorys siłowni'!$A$2:$A$18,A14)</x:f>
-        <x:v>24378.36</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$27,'Kosztorys siłowni'!$A$2:$A$27,A14)</x:f>
+        <x:v>36710.76</x:v>
       </x:c>
       <x:c r="D14" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$18,'Kosztorys siłowni'!$A$2:$A$18,A14)</x:f>
-        <x:v>29254.032</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$27,'Kosztorys siłowni'!$A$2:$A$27,A14)</x:f>
+        <x:v>44052.912</x:v>
       </x:c>
       <x:c r="E14" s="15" t="n">
         <x:f>D14/$B$7</x:f>
-        <x:v>0.20824886713281218</x:v>
+        <x:v>0.237413435783097</x:v>
       </x:c>
       <x:c r="F14" s="6" t="str"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="6" t="str">
-        <x:v>Hantle</x:v>
+        <x:v>Maszyny na nogi</x:v>
       </x:c>
       <x:c r="B15" s="6" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C15" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$18,'Kosztorys siłowni'!$A$2:$A$18,A15)</x:f>
-        <x:v>8241.58</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$27,'Kosztorys siłowni'!$A$2:$A$27,A15)</x:f>
+        <x:v>30662.57</x:v>
       </x:c>
       <x:c r="D15" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$18,'Kosztorys siłowni'!$A$2:$A$18,A15)</x:f>
-        <x:v>9889.895999999999</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$27,'Kosztorys siłowni'!$A$2:$A$27,A15)</x:f>
+        <x:v>36795.084</x:v>
       </x:c>
       <x:c r="E15" s="15" t="n">
         <x:f>D15/$B$7</x:f>
-        <x:v>0.07040259059200217</x:v>
+        <x:v>0.19829897538595545</x:v>
       </x:c>
       <x:c r="F15" s="6" t="str"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="6" t="str">
-        <x:v>Cardio</x:v>
+        <x:v>Ławki i gryfy</x:v>
       </x:c>
       <x:c r="B16" s="6" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="C16" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$18,'Kosztorys siłowni'!$A$2:$A$18,A16)</x:f>
-        <x:v>27625.239999999998</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$27,'Kosztorys siłowni'!$A$2:$A$27,A16)</x:f>
+        <x:v>5002.5599999999995</x:v>
       </x:c>
       <x:c r="D16" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$18,'Kosztorys siłowni'!$A$2:$A$18,A16)</x:f>
-        <x:v>33150.288</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$27,'Kosztorys siłowni'!$A$2:$A$27,A16)</x:f>
+        <x:v>6003.072</x:v>
       </x:c>
       <x:c r="E16" s="15" t="n">
         <x:f>D16/$B$7</x:f>
-        <x:v>0.235984903589579</x:v>
+        <x:v>0.032352230172055546</x:v>
       </x:c>
       <x:c r="F16" s="6" t="str"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="6" t="str">
-        <x:v>Drabinki i drobny sprzęt</x:v>
+        <x:v>Hantle</x:v>
       </x:c>
       <x:c r="B17" s="6" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C17" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$18,'Kosztorys siłowni'!$A$2:$A$18,A17)</x:f>
-        <x:v>5642.42</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$27,'Kosztorys siłowni'!$A$2:$A$27,A17)</x:f>
+        <x:v>8241.58</x:v>
       </x:c>
       <x:c r="D17" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$18,'Kosztorys siłowni'!$A$2:$A$18,A17)</x:f>
-        <x:v>6770.9039999999995</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$27,'Kosztorys siłowni'!$A$2:$A$27,A17)</x:f>
+        <x:v>9889.895999999999</x:v>
       </x:c>
       <x:c r="E17" s="15" t="n">
         <x:f>D17/$B$7</x:f>
-        <x:v>0.04819961526893204</x:v>
+        <x:v>0.05329940933070458</x:v>
       </x:c>
       <x:c r="F17" s="6" t="str"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="6" t="str">
-        <x:v>Wyposażenie AV</x:v>
+        <x:v>Cardio</x:v>
       </x:c>
       <x:c r="B18" s="6" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="C18" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$18,'Kosztorys siłowni'!$A$2:$A$18,A18)</x:f>
-        <x:v>8066</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$27,'Kosztorys siłowni'!$A$2:$A$27,A18)</x:f>
+        <x:v>27625.239999999998</x:v>
       </x:c>
       <x:c r="D18" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$18,'Kosztorys siłowni'!$A$2:$A$18,A18)</x:f>
-        <x:v>9679.2</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$27,'Kosztorys siłowni'!$A$2:$A$27,A18)</x:f>
+        <x:v>33150.288</x:v>
       </x:c>
       <x:c r="E18" s="15" t="n">
         <x:f>D18/$B$7</x:f>
-        <x:v>0.06890272201629902</x:v>
+        <x:v>0.17865615265749452</x:v>
       </x:c>
       <x:c r="F18" s="6" t="str"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="6" t="str">
+        <x:v>Drabinki i drobny sprzęt</x:v>
+      </x:c>
+      <x:c r="B19" s="6" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C19" s="10" t="n">
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$27,'Kosztorys siłowni'!$A$2:$A$27,A19)</x:f>
+        <x:v>5722.41</x:v>
+      </x:c>
+      <x:c r="D19" s="10" t="n">
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$27,'Kosztorys siłowni'!$A$2:$A$27,A19)</x:f>
+        <x:v>6866.892</x:v>
+      </x:c>
+      <x:c r="E19" s="15" t="n">
+        <x:f>D19/$B$7</x:f>
+        <x:v>0.037007597202007046</x:v>
+      </x:c>
+      <x:c r="F19" s="6" t="str"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="6" t="str">
+        <x:v>Opcjonalne uzupełnienie</x:v>
+      </x:c>
+      <x:c r="B20" s="6" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C20" s="10" t="n">
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$27,'Kosztorys siłowni'!$A$2:$A$27,A20)</x:f>
+        <x:v>3005.95</x:v>
+      </x:c>
+      <x:c r="D20" s="10" t="n">
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$27,'Kosztorys siłowni'!$A$2:$A$27,A20)</x:f>
+        <x:v>3607.1399999999994</x:v>
+      </x:c>
+      <x:c r="E20" s="15" t="n">
+        <x:f>D20/$B$7</x:f>
+        <x:v>0.01943988403651138</x:v>
+      </x:c>
+      <x:c r="F20" s="6" t="str"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="6" t="str">
+        <x:v>Wyposażenie AV</x:v>
+      </x:c>
+      <x:c r="B21" s="6" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C21" s="10" t="n">
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$27,'Kosztorys siłowni'!$A$2:$A$27,A21)</x:f>
+        <x:v>8066</x:v>
+      </x:c>
+      <x:c r="D21" s="10" t="n">
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$27,'Kosztorys siłowni'!$A$2:$A$27,A21)</x:f>
+        <x:v>9679.2</x:v>
+      </x:c>
+      <x:c r="E21" s="15" t="n">
+        <x:f>D21/$B$7</x:f>
+        <x:v>0.052163909791746635</x:v>
+      </x:c>
+      <x:c r="F21" s="6" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -731,396 +794,648 @@
         <x:v>Wolne ciężary</x:v>
       </x:c>
       <x:c r="B6" s="19" t="str">
-        <x:v>Osłona na gryf PROUD Barbell Pad</x:v>
+        <x:v>Obciążenie olimpijskie Fractional Competition PROUD 0,5-2,5 kg</x:v>
       </x:c>
       <x:c r="C6" s="6" t="str">
-        <x:v>1</x:v>
+        <x:v>1 zestaw</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>62.61</x:v>
+        <x:v>749.99</x:v>
       </x:c>
       <x:c r="E6" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F6" s="10" t="n">
         <x:f>D6</x:f>
-        <x:v>62.61</x:v>
+        <x:v>749.99</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
         <x:f>F6*(1+E6)</x:f>
-        <x:v>75.13199999999999</x:v>
+        <x:v>899.9879999999999</x:v>
       </x:c>
       <x:c r="H6" s="19" t="str">
-        <x:v>https://trainingshowroom.com/akcesoria/2488-ochraniacz-na-gryf-proud-barbell-pad.html</x:v>
+        <x:v>https://trainingshowroom.com/talerze/2335-zestaw-obciazen-olimpijskich-proud-competition-fractional-plate.html</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="6" t="str">
-        <x:v>Maszyny siłowe</x:v>
+        <x:v>Wolne ciężary</x:v>
       </x:c>
       <x:c r="B7" s="19" t="str">
-        <x:v>Wyciąg górny / dolny PROUD Champion Outlet</x:v>
+        <x:v>Osłona na gryf PROUD Barbell Pad</x:v>
       </x:c>
       <x:c r="C7" s="6" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>15081.31</x:v>
+        <x:v>62.61</x:v>
       </x:c>
       <x:c r="E7" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F7" s="10" t="n">
         <x:f>D7</x:f>
-        <x:v>15081.31</x:v>
+        <x:v>62.61</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
         <x:f>F7*(1+E7)</x:f>
-        <x:v>18097.572</x:v>
+        <x:v>75.13199999999999</x:v>
       </x:c>
       <x:c r="H7" s="19" t="str">
-        <x:v>https://trainingshowroom.com/outlet/3506-wyciag-gorny-wyciag-dolny-proud-champion-outlet.html</x:v>
+        <x:v>https://trainingshowroom.com/akcesoria/2488-ochraniacz-na-gryf-proud-barbell-pad.html</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="6" t="str">
-        <x:v>Maszyny siłowe</x:v>
+        <x:v>Przechowywanie</x:v>
       </x:c>
       <x:c r="B8" s="19" t="str">
-        <x:v>Podwójny uchwyt do wyciągu, trójkąt PROUD</x:v>
+        <x:v>Stojak na obciążenia i gryfy olimpijskie PROUD</x:v>
       </x:c>
       <x:c r="C8" s="6" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>109.07</x:v>
+        <x:v>921.31</x:v>
       </x:c>
       <x:c r="E8" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F8" s="10" t="n">
         <x:f>D8</x:f>
-        <x:v>109.07</x:v>
+        <x:v>921.31</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
         <x:f>F8*(1+E8)</x:f>
-        <x:v>130.884</x:v>
+        <x:v>1105.572</x:v>
       </x:c>
       <x:c r="H8" s="19" t="str">
-        <x:v>https://trainingshowroom.com/maszyny-silowe/2581-podwojny-uchwyt-do-wyciagu-ogumowany-trojkat-proud.html</x:v>
+        <x:v>https://trainingshowroom.com/outlet/2373-stojak-na-obciazenia-i-gryfy-olimpijskie-proud.html</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="6" t="str">
-        <x:v>Maszyny na nogi</x:v>
+        <x:v>Maszyny siłowe</x:v>
       </x:c>
       <x:c r="B9" s="19" t="str">
-        <x:v>Maszyna do przysiadów Hack PROUD Champion</x:v>
+        <x:v>Wyciąg górny / dolny PROUD Champion Outlet</x:v>
       </x:c>
       <x:c r="C9" s="6" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>13269.37</x:v>
+        <x:v>15081.31</x:v>
       </x:c>
       <x:c r="E9" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F9" s="10" t="n">
         <x:f>D9</x:f>
-        <x:v>13269.37</x:v>
+        <x:v>15081.31</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
         <x:f>F9*(1+E9)</x:f>
-        <x:v>15923.244</x:v>
+        <x:v>18097.572</x:v>
       </x:c>
       <x:c r="H9" s="19" t="str">
-        <x:v>https://trainingshowroom.com/maszyny-silowe/2939-maszyna-do-przysiadow-proud-champion.html</x:v>
+        <x:v>https://trainingshowroom.com/outlet/3506-wyciag-gorny-wyciag-dolny-proud-champion-outlet.html</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="6" t="str">
-        <x:v>Maszyny na nogi</x:v>
+        <x:v>Maszyny siłowe</x:v>
       </x:c>
       <x:c r="B10" s="19" t="str">
-        <x:v>Seated Leg Extension Plate Loaded PROUD Champion</x:v>
+        <x:v>Podwójny uchwyt do wyciągu, trójkąt PROUD</x:v>
       </x:c>
       <x:c r="C10" s="6" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>11108.99</x:v>
+        <x:v>109.07</x:v>
       </x:c>
       <x:c r="E10" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F10" s="10" t="n">
         <x:f>D10</x:f>
-        <x:v>11108.99</x:v>
+        <x:v>109.07</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
         <x:f>F10*(1+E10)</x:f>
-        <x:v>13330.787999999999</x:v>
+        <x:v>130.884</x:v>
       </x:c>
       <x:c r="H10" s="19" t="str">
-        <x:v>https://trainingshowroom.com/maszyny-na-wolny-ciezar/3404-maszyna-seated-leg-extension-plate-loaded-proud-champion.html</x:v>
+        <x:v>https://trainingshowroom.com/maszyny-silowe/2581-podwojny-uchwyt-do-wyciagu-ogumowany-trojkat-proud.html</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="6" t="str">
-        <x:v>Hantle</x:v>
+        <x:v>Maszyny siłowe</x:v>
       </x:c>
       <x:c r="B11" s="19" t="str">
-        <x:v>Hantle poliuretanowe Studio PROUD, zestaw 1-10 kg</x:v>
+        <x:v>Wyciąg regulowany Dual Pulley PROUD Champion</x:v>
       </x:c>
       <x:c r="C11" s="6" t="str">
-        <x:v>2 zestawy</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>8241.58</x:v>
+        <x:v>21520.38</x:v>
       </x:c>
       <x:c r="E11" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F11" s="10" t="n">
         <x:f>D11</x:f>
-        <x:v>8241.58</x:v>
+        <x:v>21520.38</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
         <x:f>F11*(1+E11)</x:f>
-        <x:v>9889.895999999999</x:v>
+        <x:v>25824.456000000002</x:v>
       </x:c>
       <x:c r="H11" s="19" t="str">
-        <x:v>https://trainingshowroom.com/hantle-i-kettlebells/3467-hantle-poliuretanowe-studio-zestaw-proud.html</x:v>
+        <x:v>https://trainingshowroom.com/maszyny-silowe/2906-wyciag-regulowany-dual-pulley-proud-champion.html</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="6" t="str">
-        <x:v>Cardio</x:v>
+        <x:v>Maszyny na nogi</x:v>
       </x:c>
       <x:c r="B12" s="19" t="str">
-        <x:v>Ergometr wioślarski AIR 2.0 PROUD</x:v>
+        <x:v>Maszyna do przysiadów Hack PROUD Champion</x:v>
       </x:c>
       <x:c r="C12" s="6" t="str">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D12" s="10" t="n">
-        <x:v>10720.12</x:v>
+        <x:v>13269.37</x:v>
       </x:c>
       <x:c r="E12" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F12" s="10" t="n">
         <x:f>D12</x:f>
-        <x:v>10720.12</x:v>
+        <x:v>13269.37</x:v>
       </x:c>
       <x:c r="G12" s="10" t="n">
         <x:f>F12*(1+E12)</x:f>
-        <x:v>12864.144</x:v>
+        <x:v>15923.244</x:v>
       </x:c>
       <x:c r="H12" s="19" t="str">
-        <x:v>https://trainingshowroom.com/ergometry/2782-ergometr-wioslarski-air-proud-20.html?hsCtaAttrib=186811937891</x:v>
+        <x:v>https://trainingshowroom.com/maszyny-silowe/2939-maszyna-do-przysiadow-proud-champion.html</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="6" t="str">
-        <x:v>Cardio</x:v>
+        <x:v>Maszyny na nogi</x:v>
       </x:c>
       <x:c r="B13" s="19" t="str">
-        <x:v>Air Runner, bieżnia treningowa 2.0 Elite PROUD Outlet</x:v>
+        <x:v>Seated Leg Extension Plate Loaded PROUD Champion</x:v>
       </x:c>
       <x:c r="C13" s="6" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D13" s="10" t="n">
-        <x:v>16905.12</x:v>
+        <x:v>11108.99</x:v>
       </x:c>
       <x:c r="E13" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F13" s="10" t="n">
         <x:f>D13</x:f>
-        <x:v>16905.12</x:v>
+        <x:v>11108.99</x:v>
       </x:c>
       <x:c r="G13" s="10" t="n">
         <x:f>F13*(1+E13)</x:f>
-        <x:v>20286.143999999997</x:v>
+        <x:v>13330.787999999999</x:v>
       </x:c>
       <x:c r="H13" s="19" t="str">
-        <x:v>https://trainingshowroom.com/bieznie/3501-air-runner-bieznia-treningowa-20-elite-proud-outlet.html</x:v>
+        <x:v>https://trainingshowroom.com/maszyny-na-wolny-ciezar/3404-maszyna-seated-leg-extension-plate-loaded-proud-champion.html</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="6" t="str">
-        <x:v>Drabinki i drobny sprzęt</x:v>
+        <x:v>Maszyny na nogi</x:v>
       </x:c>
       <x:c r="B14" s="19" t="str">
-        <x:v>Poręcze do drabinki PROUD Champion Outlet</x:v>
+        <x:v>Maszyna do treningu łydek PROUD Champion</x:v>
       </x:c>
       <x:c r="C14" s="6" t="str">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D14" s="10" t="n">
-        <x:v>2451.86</x:v>
+        <x:v>6284.21</x:v>
       </x:c>
       <x:c r="E14" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F14" s="10" t="n">
         <x:f>D14</x:f>
-        <x:v>2451.86</x:v>
+        <x:v>6284.21</x:v>
       </x:c>
       <x:c r="G14" s="10" t="n">
         <x:f>F14*(1+E14)</x:f>
-        <x:v>2942.232</x:v>
+        <x:v>7541.052</x:v>
       </x:c>
       <x:c r="H14" s="19" t="str">
-        <x:v>https://trainingshowroom.com/outlet/3584-porecze-do-drabinki-proud-champion-outlet.html</x:v>
+        <x:v>https://trainingshowroom.com/maszyny-silowe/2938-maszyna-do-lydek-proud-champion.html</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="6" t="str">
-        <x:v>Drabinki i drobny sprzęt</x:v>
+        <x:v>Ławki i gryfy</x:v>
       </x:c>
       <x:c r="B15" s="19" t="str">
-        <x:v>Drabinka gimnastyczna PROUD</x:v>
+        <x:v>Modlitewnik PROUD Champion</x:v>
       </x:c>
       <x:c r="C15" s="6" t="str">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D15" s="10" t="n">
-        <x:v>1939.18</x:v>
+        <x:v>4502.57</x:v>
       </x:c>
       <x:c r="E15" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F15" s="10" t="n">
         <x:f>D15</x:f>
-        <x:v>1939.18</x:v>
+        <x:v>4502.57</x:v>
       </x:c>
       <x:c r="G15" s="10" t="n">
         <x:f>F15*(1+E15)</x:f>
-        <x:v>2327.016</x:v>
+        <x:v>5403.084</x:v>
       </x:c>
       <x:c r="H15" s="19" t="str">
-        <x:v>https://trainingshowroom.com/sprzet-gimnastyczny/2272-drabinka-gimnastyczna-proud.html</x:v>
+        <x:v>https://trainingshowroom.com/champion/2970-modlitewnik-proud-champion.html?search_query=Modlitewnik</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="6" t="str">
-        <x:v>Drabinki i drobny sprzęt</x:v>
+        <x:v>Ławki i gryfy</x:v>
       </x:c>
       <x:c r="B16" s="19" t="str">
-        <x:v>Drążek do podciągania do drabinki PROUD Champion Outlet</x:v>
+        <x:v>Gryf olimpijski treningowy łamany Curl Silver PROUD</x:v>
       </x:c>
       <x:c r="C16" s="6" t="str">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D16" s="10" t="n">
-        <x:v>1251.38</x:v>
+        <x:v>499.99</x:v>
       </x:c>
       <x:c r="E16" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F16" s="10" t="n">
         <x:f>D16</x:f>
-        <x:v>1251.38</x:v>
+        <x:v>499.99</x:v>
       </x:c>
       <x:c r="G16" s="10" t="n">
         <x:f>F16*(1+E16)</x:f>
-        <x:v>1501.6560000000002</x:v>
+        <x:v>599.9879999999999</x:v>
       </x:c>
       <x:c r="H16" s="19" t="str">
-        <x:v>https://trainingshowroom.com/outlet/3585-drazek-do-podciagania-do-drabinki-proud-champion-outlet.html</x:v>
+        <x:v>https://trainingshowroom.com/sztangi/2596-gryf-olimpijski-treningowy-lamany-silver-proud.html</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="6" t="str">
-        <x:v>Wyposażenie AV</x:v>
+        <x:v>Hantle</x:v>
       </x:c>
       <x:c r="B17" s="19" t="str">
-        <x:v>Projektor Full HD Epson EB-FH52</x:v>
+        <x:v>Hantle poliuretanowe Studio PROUD, zestaw 1-10 kg</x:v>
       </x:c>
       <x:c r="C17" s="6" t="str">
-        <x:v>1</x:v>
+        <x:v>2 zestawy</x:v>
       </x:c>
       <x:c r="D17" s="10" t="n">
-        <x:v>4559</x:v>
+        <x:v>8241.58</x:v>
       </x:c>
       <x:c r="E17" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F17" s="10" t="n">
         <x:f>D17</x:f>
-        <x:v>4559</x:v>
+        <x:v>8241.58</x:v>
       </x:c>
       <x:c r="G17" s="10" t="n">
         <x:f>F17*(1+E17)</x:f>
-        <x:v>5470.8</x:v>
+        <x:v>9889.895999999999</x:v>
       </x:c>
       <x:c r="H17" s="19" t="str">
-        <x:v>https://www.x-kom.pl/p/1224184-projektor-epson-eb-fh52.html</x:v>
+        <x:v>https://trainingshowroom.com/hantle-i-kettlebells/3467-hantle-poliuretanowe-studio-zestaw-proud.html</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="6" t="str">
-        <x:v>Wyposażenie AV</x:v>
+        <x:v>Cardio</x:v>
       </x:c>
       <x:c r="B18" s="19" t="str">
-        <x:v>Mobilny zestaw audio LD Systems Roadbuddy 10 HHD 2</x:v>
+        <x:v>Ergometr wioślarski AIR 2.0 PROUD</x:v>
       </x:c>
       <x:c r="C18" s="6" t="str">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D18" s="10" t="n">
-        <x:v>3507</x:v>
+        <x:v>10720.12</x:v>
       </x:c>
       <x:c r="E18" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F18" s="10" t="n">
         <x:f>D18</x:f>
-        <x:v>3507</x:v>
+        <x:v>10720.12</x:v>
       </x:c>
       <x:c r="G18" s="10" t="n">
         <x:f>F18*(1+E18)</x:f>
+        <x:v>12864.144</x:v>
+      </x:c>
+      <x:c r="H18" s="19" t="str">
+        <x:v>https://trainingshowroom.com/ergometry/2782-ergometr-wioslarski-air-proud-20.html?hsCtaAttrib=186811937891</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="6" t="str">
+        <x:v>Cardio</x:v>
+      </x:c>
+      <x:c r="B19" s="19" t="str">
+        <x:v>Air Runner, bieżnia treningowa 2.0 Elite PROUD Outlet</x:v>
+      </x:c>
+      <x:c r="C19" s="6" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D19" s="10" t="n">
+        <x:v>16905.12</x:v>
+      </x:c>
+      <x:c r="E19" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F19" s="10" t="n">
+        <x:f>D19</x:f>
+        <x:v>16905.12</x:v>
+      </x:c>
+      <x:c r="G19" s="10" t="n">
+        <x:f>F19*(1+E19)</x:f>
+        <x:v>20286.143999999997</x:v>
+      </x:c>
+      <x:c r="H19" s="19" t="str">
+        <x:v>https://trainingshowroom.com/bieznie/3501-air-runner-bieznia-treningowa-20-elite-proud-outlet.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="6" t="str">
+        <x:v>Drabinki i drobny sprzęt</x:v>
+      </x:c>
+      <x:c r="B20" s="19" t="str">
+        <x:v>Poręcze do drabinki PROUD Champion Outlet</x:v>
+      </x:c>
+      <x:c r="C20" s="6" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D20" s="10" t="n">
+        <x:v>2451.86</x:v>
+      </x:c>
+      <x:c r="E20" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F20" s="10" t="n">
+        <x:f>D20</x:f>
+        <x:v>2451.86</x:v>
+      </x:c>
+      <x:c r="G20" s="10" t="n">
+        <x:f>F20*(1+E20)</x:f>
+        <x:v>2942.232</x:v>
+      </x:c>
+      <x:c r="H20" s="19" t="str">
+        <x:v>https://trainingshowroom.com/outlet/3584-porecze-do-drabinki-proud-champion-outlet.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="6" t="str">
+        <x:v>Drabinki i drobny sprzęt</x:v>
+      </x:c>
+      <x:c r="B21" s="19" t="str">
+        <x:v>Drabinka gimnastyczna PROUD</x:v>
+      </x:c>
+      <x:c r="C21" s="6" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D21" s="10" t="n">
+        <x:v>1939.18</x:v>
+      </x:c>
+      <x:c r="E21" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F21" s="10" t="n">
+        <x:f>D21</x:f>
+        <x:v>1939.18</x:v>
+      </x:c>
+      <x:c r="G21" s="10" t="n">
+        <x:f>F21*(1+E21)</x:f>
+        <x:v>2327.016</x:v>
+      </x:c>
+      <x:c r="H21" s="19" t="str">
+        <x:v>https://trainingshowroom.com/sprzet-gimnastyczny/2272-drabinka-gimnastyczna-proud.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="6" t="str">
+        <x:v>Drabinki i drobny sprzęt</x:v>
+      </x:c>
+      <x:c r="B22" s="19" t="str">
+        <x:v>Drążek do podciągania do drabinki PROUD Champion Outlet</x:v>
+      </x:c>
+      <x:c r="C22" s="6" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D22" s="10" t="n">
+        <x:v>1251.38</x:v>
+      </x:c>
+      <x:c r="E22" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F22" s="10" t="n">
+        <x:f>D22</x:f>
+        <x:v>1251.38</x:v>
+      </x:c>
+      <x:c r="G22" s="10" t="n">
+        <x:f>F22*(1+E22)</x:f>
+        <x:v>1501.6560000000002</x:v>
+      </x:c>
+      <x:c r="H22" s="19" t="str">
+        <x:v>https://trainingshowroom.com/outlet/3585-drazek-do-podciagania-do-drabinki-proud-champion-outlet.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="6" t="str">
+        <x:v>Drabinki i drobny sprzęt</x:v>
+      </x:c>
+      <x:c r="B23" s="19" t="str">
+        <x:v>Podkładki do przysiadów PROUD</x:v>
+      </x:c>
+      <x:c r="C23" s="6" t="str">
+        <x:v>1 komplet</x:v>
+      </x:c>
+      <x:c r="D23" s="10" t="n">
+        <x:v>79.99</x:v>
+      </x:c>
+      <x:c r="E23" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F23" s="10" t="n">
+        <x:f>D23</x:f>
+        <x:v>79.99</x:v>
+      </x:c>
+      <x:c r="G23" s="10" t="n">
+        <x:f>F23*(1+E23)</x:f>
+        <x:v>95.98799999999999</x:v>
+      </x:c>
+      <x:c r="H23" s="19" t="str">
+        <x:v>https://trainingshowroom.com/gumy-i-rollery/3356-podkladki-do-przysiadow-proud.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="6" t="str">
+        <x:v>Opcjonalne uzupełnienie</x:v>
+      </x:c>
+      <x:c r="B24" s="19" t="str">
+        <x:v>Kettlebell żeliwny PRO, zestaw PROUD</x:v>
+      </x:c>
+      <x:c r="C24" s="6" t="str">
+        <x:v>1 zestaw</x:v>
+      </x:c>
+      <x:c r="D24" s="10" t="n">
+        <x:v>2625.99</x:v>
+      </x:c>
+      <x:c r="E24" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F24" s="10" t="n">
+        <x:f>D24</x:f>
+        <x:v>2625.99</x:v>
+      </x:c>
+      <x:c r="G24" s="10" t="n">
+        <x:f>F24*(1+E24)</x:f>
+        <x:v>3151.1879999999996</x:v>
+      </x:c>
+      <x:c r="H24" s="19" t="str">
+        <x:v>https://trainingshowroom.com/hantle-i-kettlebells/3465-hantla-proud-kettlebell-zestaw.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="6" t="str">
+        <x:v>Opcjonalne uzupełnienie</x:v>
+      </x:c>
+      <x:c r="B25" s="19" t="str">
+        <x:v>Podłoga gumowa Standard PROUD pod kettlebell</x:v>
+      </x:c>
+      <x:c r="C25" s="6" t="str">
+        <x:v>4 szt.</x:v>
+      </x:c>
+      <x:c r="D25" s="10" t="n">
+        <x:v>379.96</x:v>
+      </x:c>
+      <x:c r="E25" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F25" s="10" t="n">
+        <x:f>D25</x:f>
+        <x:v>379.96</x:v>
+      </x:c>
+      <x:c r="G25" s="10" t="n">
+        <x:f>F25*(1+E25)</x:f>
+        <x:v>455.95199999999994</x:v>
+      </x:c>
+      <x:c r="H25" s="19" t="str">
+        <x:v>https://trainingshowroom.com/podlogi/3427-podloga-gumowa-standard-proud.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="6" t="str">
+        <x:v>Wyposażenie AV</x:v>
+      </x:c>
+      <x:c r="B26" s="19" t="str">
+        <x:v>Projektor Full HD Epson EB-FH52</x:v>
+      </x:c>
+      <x:c r="C26" s="6" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D26" s="10" t="n">
+        <x:v>4559</x:v>
+      </x:c>
+      <x:c r="E26" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F26" s="10" t="n">
+        <x:f>D26</x:f>
+        <x:v>4559</x:v>
+      </x:c>
+      <x:c r="G26" s="10" t="n">
+        <x:f>F26*(1+E26)</x:f>
+        <x:v>5470.8</x:v>
+      </x:c>
+      <x:c r="H26" s="19" t="str">
+        <x:v>https://www.x-kom.pl/p/1224184-projektor-epson-eb-fh52.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="6" t="str">
+        <x:v>Wyposażenie AV</x:v>
+      </x:c>
+      <x:c r="B27" s="19" t="str">
+        <x:v>Mobilny zestaw audio LD Systems Roadbuddy 10 HHD 2</x:v>
+      </x:c>
+      <x:c r="C27" s="6" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D27" s="10" t="n">
+        <x:v>3507</x:v>
+      </x:c>
+      <x:c r="E27" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F27" s="10" t="n">
+        <x:f>D27</x:f>
+        <x:v>3507</x:v>
+      </x:c>
+      <x:c r="G27" s="10" t="n">
+        <x:f>F27*(1+E27)</x:f>
         <x:v>4208.4</x:v>
       </x:c>
-      <x:c r="H18" s="19" t="str">
+      <x:c r="H27" s="19" t="str">
         <x:v>https://www.ceneo.pl/89383056</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="6"/>
-      <x:c r="B19" s="6"/>
-      <x:c r="C19" s="6"/>
-      <x:c r="D19" s="10"/>
-      <x:c r="E19" s="6"/>
-      <x:c r="F19" s="10"/>
-      <x:c r="G19" s="10"/>
-      <x:c r="H19" s="6"/>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="17" t="str">
+    <x:row r="28">
+      <x:c r="A28" s="6"/>
+      <x:c r="B28" s="6"/>
+      <x:c r="C28" s="6"/>
+      <x:c r="D28" s="10"/>
+      <x:c r="E28" s="6"/>
+      <x:c r="F28" s="10"/>
+      <x:c r="G28" s="10"/>
+      <x:c r="H28" s="6"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="17" t="str">
         <x:v>Razem</x:v>
       </x:c>
-      <x:c r="B20" s="17"/>
-      <x:c r="C20" s="17"/>
-      <x:c r="D20" s="18"/>
-      <x:c r="E20" s="17"/>
-      <x:c r="F20" s="18" t="n">
-        <x:f>SUM(F2:F18)</x:f>
-        <x:v>117063.59</x:v>
-      </x:c>
-      <x:c r="G20" s="18" t="n">
-        <x:f>SUM(G2:G18)</x:f>
-        <x:v>140476.308</x:v>
-      </x:c>
-      <x:c r="H20" s="17"/>
+      <x:c r="B29" s="17"/>
+      <x:c r="C29" s="17"/>
+      <x:c r="D29" s="18"/>
+      <x:c r="E29" s="17"/>
+      <x:c r="F29" s="18" t="n">
+        <x:f>SUM(F2:F27)</x:f>
+        <x:v>154627.97999999995</x:v>
+      </x:c>
+      <x:c r="G29" s="18" t="n">
+        <x:f>SUM(G2:G27)</x:f>
+        <x:v>185553.57599999994</x:v>
+      </x:c>
+      <x:c r="H29" s="17"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A20:C20"/>
+    <x:mergeCell ref="A29:C29"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Update AV equipment and add gym machines
</commit_message>
<xml_diff>
--- a/outputs/wyposazenie-silowni/wyposazenie-silowni-zsz5-2027.xlsx
+++ b/outputs/wyposazenie-silowni/wyposazenie-silowni-zsz5-2027.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Podsumowanie" sheetId="1" r:id="Rf3b5b6b067744a7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kosztorys siłowni" sheetId="2" r:id="Ra973be4e75454619"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Podsumowanie" sheetId="1" r:id="Rbc6db7a558bb4d08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kosztorys siłowni" sheetId="2" r:id="R51aa0fdbf3c94daf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -348,7 +348,7 @@
         <x:v>Liczba pozycji</x:v>
       </x:c>
       <x:c r="B4" s="6" t="n">
-        <x:v>26</x:v>
+        <x:v>34</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -364,8 +364,8 @@
         <x:v>Suma cen sprzętu</x:v>
       </x:c>
       <x:c r="B6" s="10" t="n">
-        <x:f>'Kosztorys siłowni'!F29</x:f>
-        <x:v>154627.97999999995</x:v>
+        <x:f>'Kosztorys siłowni'!F37</x:f>
+        <x:v>191955.24</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -373,8 +373,8 @@
         <x:v>Prognozowana suma +20%</x:v>
       </x:c>
       <x:c r="B7" s="12" t="n">
-        <x:f>'Kosztorys siłowni'!G29</x:f>
-        <x:v>185553.57599999994</x:v>
+        <x:f>'Kosztorys siłowni'!G37</x:f>
+        <x:v>230346.2879999999</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -405,16 +405,16 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$27,'Kosztorys siłowni'!$A$2:$A$27,A11)</x:f>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A11)</x:f>
         <x:v>16297</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$27,'Kosztorys siłowni'!$A$2:$A$27,A11)</x:f>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A11)</x:f>
         <x:v>19556.399999999998</x:v>
       </x:c>
       <x:c r="E11" s="15" t="n">
         <x:f>D11/$B$7</x:f>
-        <x:v>0.105394896835618</x:v>
+        <x:v>0.08490000064598395</x:v>
       </x:c>
       <x:c r="F11" s="6" t="str"/>
     </x:row>
@@ -426,16 +426,16 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C12" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$27,'Kosztorys siłowni'!$A$2:$A$27,A12)</x:f>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A12)</x:f>
         <x:v>12372.6</x:v>
       </x:c>
       <x:c r="D12" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$27,'Kosztorys siłowni'!$A$2:$A$27,A12)</x:f>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A12)</x:f>
         <x:v>14847.119999999999</x:v>
       </x:c>
       <x:c r="E12" s="15" t="n">
         <x:f>D12/$B$7</x:f>
-        <x:v>0.08001527278568861</x:v>
+        <x:v>0.06445565122369154</x:v>
       </x:c>
       <x:c r="F12" s="6" t="str"/>
     </x:row>
@@ -447,16 +447,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C13" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$27,'Kosztorys siłowni'!$A$2:$A$27,A13)</x:f>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A13)</x:f>
         <x:v>921.31</x:v>
       </x:c>
       <x:c r="D13" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$27,'Kosztorys siłowni'!$A$2:$A$27,A13)</x:f>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A13)</x:f>
         <x:v>1105.572</x:v>
       </x:c>
       <x:c r="E13" s="15" t="n">
         <x:f>D13/$B$7</x:f>
-        <x:v>0.005958236019121509</x:v>
+        <x:v>0.004799608492063047</x:v>
       </x:c>
       <x:c r="F13" s="6" t="str"/>
     </x:row>
@@ -465,168 +465,189 @@
         <x:v>Maszyny siłowe</x:v>
       </x:c>
       <x:c r="B14" s="6" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C14" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$27,'Kosztorys siłowni'!$A$2:$A$27,A14)</x:f>
-        <x:v>36710.76</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A14)</x:f>
+        <x:v>56851.16</x:v>
       </x:c>
       <x:c r="D14" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$27,'Kosztorys siłowni'!$A$2:$A$27,A14)</x:f>
-        <x:v>44052.912</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A14)</x:f>
+        <x:v>68221.39199999999</x:v>
       </x:c>
       <x:c r="E14" s="15" t="n">
         <x:f>D14/$B$7</x:f>
-        <x:v>0.237413435783097</x:v>
+        <x:v>0.29616883602656546</x:v>
       </x:c>
       <x:c r="F14" s="6" t="str"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="6" t="str">
-        <x:v>Maszyny na nogi</x:v>
+        <x:v>Maszyny na plecy</x:v>
       </x:c>
       <x:c r="B15" s="6" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C15" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$27,'Kosztorys siłowni'!$A$2:$A$27,A15)</x:f>
-        <x:v>30662.57</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A15)</x:f>
+        <x:v>8169.88</x:v>
       </x:c>
       <x:c r="D15" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$27,'Kosztorys siłowni'!$A$2:$A$27,A15)</x:f>
-        <x:v>36795.084</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A15)</x:f>
+        <x:v>9803.856</x:v>
       </x:c>
       <x:c r="E15" s="15" t="n">
         <x:f>D15/$B$7</x:f>
-        <x:v>0.19829897538595545</x:v>
+        <x:v>0.042561380455151954</x:v>
       </x:c>
       <x:c r="F15" s="6" t="str"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="6" t="str">
-        <x:v>Ławki i gryfy</x:v>
+        <x:v>Maszyny na nogi</x:v>
       </x:c>
       <x:c r="B16" s="6" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C16" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$27,'Kosztorys siłowni'!$A$2:$A$27,A16)</x:f>
-        <x:v>5002.5599999999995</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A16)</x:f>
+        <x:v>30662.57</x:v>
       </x:c>
       <x:c r="D16" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$27,'Kosztorys siłowni'!$A$2:$A$27,A16)</x:f>
-        <x:v>6003.072</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A16)</x:f>
+        <x:v>36795.084</x:v>
       </x:c>
       <x:c r="E16" s="15" t="n">
         <x:f>D16/$B$7</x:f>
-        <x:v>0.032352230172055546</x:v>
+        <x:v>0.15973812436690976</x:v>
       </x:c>
       <x:c r="F16" s="6" t="str"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="6" t="str">
-        <x:v>Hantle</x:v>
+        <x:v>Ławki i gryfy</x:v>
       </x:c>
       <x:c r="B17" s="6" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C17" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$27,'Kosztorys siłowni'!$A$2:$A$27,A17)</x:f>
-        <x:v>8241.58</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A17)</x:f>
+        <x:v>5002.5599999999995</x:v>
       </x:c>
       <x:c r="D17" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$27,'Kosztorys siłowni'!$A$2:$A$27,A17)</x:f>
-        <x:v>9889.895999999999</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A17)</x:f>
+        <x:v>6003.072</x:v>
       </x:c>
       <x:c r="E17" s="15" t="n">
         <x:f>D17/$B$7</x:f>
-        <x:v>0.05329940933070458</x:v>
+        <x:v>0.0260610754882232</x:v>
       </x:c>
       <x:c r="F17" s="6" t="str"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="6" t="str">
-        <x:v>Cardio</x:v>
+        <x:v>Hantle</x:v>
       </x:c>
       <x:c r="B18" s="6" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C18" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$27,'Kosztorys siłowni'!$A$2:$A$27,A18)</x:f>
-        <x:v>27625.239999999998</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A18)</x:f>
+        <x:v>8241.58</x:v>
       </x:c>
       <x:c r="D18" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$27,'Kosztorys siłowni'!$A$2:$A$27,A18)</x:f>
-        <x:v>33150.288</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A18)</x:f>
+        <x:v>9889.895999999999</x:v>
       </x:c>
       <x:c r="E18" s="15" t="n">
         <x:f>D18/$B$7</x:f>
-        <x:v>0.17865615265749452</x:v>
+        <x:v>0.04293490503306918</x:v>
       </x:c>
       <x:c r="F18" s="6" t="str"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="6" t="str">
-        <x:v>Drabinki i drobny sprzęt</x:v>
+        <x:v>Cardio</x:v>
       </x:c>
       <x:c r="B19" s="6" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C19" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$27,'Kosztorys siłowni'!$A$2:$A$27,A19)</x:f>
-        <x:v>5722.41</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A19)</x:f>
+        <x:v>27625.239999999998</x:v>
       </x:c>
       <x:c r="D19" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$27,'Kosztorys siłowni'!$A$2:$A$27,A19)</x:f>
-        <x:v>6866.892</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A19)</x:f>
+        <x:v>33150.288</x:v>
       </x:c>
       <x:c r="E19" s="15" t="n">
         <x:f>D19/$B$7</x:f>
-        <x:v>0.037007597202007046</x:v>
+        <x:v>0.14391500851969455</x:v>
       </x:c>
       <x:c r="F19" s="6" t="str"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="6" t="str">
-        <x:v>Opcjonalne uzupełnienie</x:v>
+        <x:v>Drabinki i drobny sprzęt</x:v>
       </x:c>
       <x:c r="B20" s="6" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C20" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$27,'Kosztorys siłowni'!$A$2:$A$27,A20)</x:f>
-        <x:v>3005.95</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A20)</x:f>
+        <x:v>5722.41</x:v>
       </x:c>
       <x:c r="D20" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$27,'Kosztorys siłowni'!$A$2:$A$27,A20)</x:f>
-        <x:v>3607.1399999999994</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A20)</x:f>
+        <x:v>6866.892</x:v>
       </x:c>
       <x:c r="E20" s="15" t="n">
         <x:f>D20/$B$7</x:f>
-        <x:v>0.01943988403651138</x:v>
+        <x:v>0.029811168478651597</x:v>
       </x:c>
       <x:c r="F20" s="6" t="str"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="6" t="str">
-        <x:v>Wyposażenie AV</x:v>
+        <x:v>Opcjonalne uzupełnienie</x:v>
       </x:c>
       <x:c r="B21" s="6" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="C21" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$27,'Kosztorys siłowni'!$A$2:$A$27,A21)</x:f>
-        <x:v>8066</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A21)</x:f>
+        <x:v>3005.95</x:v>
       </x:c>
       <x:c r="D21" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$27,'Kosztorys siłowni'!$A$2:$A$27,A21)</x:f>
-        <x:v>9679.2</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A21)</x:f>
+        <x:v>3607.1399999999994</x:v>
       </x:c>
       <x:c r="E21" s="15" t="n">
         <x:f>D21/$B$7</x:f>
-        <x:v>0.052163909791746635</x:v>
+        <x:v>0.01565964023696358</x:v>
       </x:c>
       <x:c r="F21" s="6" t="str"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="6" t="str">
+        <x:v>Wyposażenie AV</x:v>
+      </x:c>
+      <x:c r="B22" s="6" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C22" s="10" t="n">
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A22)</x:f>
+        <x:v>17082.98</x:v>
+      </x:c>
+      <x:c r="D22" s="10" t="n">
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A22)</x:f>
+        <x:v>20499.575999999997</x:v>
+      </x:c>
+      <x:c r="E22" s="15" t="n">
+        <x:f>D22/$B$7</x:f>
+        <x:v>0.08899460103303251</x:v>
+      </x:c>
+      <x:c r="F22" s="6" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -959,58 +980,58 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="6" t="str">
-        <x:v>Maszyny na nogi</x:v>
+        <x:v>Maszyny siłowe</x:v>
       </x:c>
       <x:c r="B12" s="19" t="str">
-        <x:v>Maszyna do przysiadów Hack PROUD Champion</x:v>
+        <x:v>Maszyna Leverage Chest Press PROUD Champion</x:v>
       </x:c>
       <x:c r="C12" s="6" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D12" s="10" t="n">
-        <x:v>13269.37</x:v>
+        <x:v>20140.4</x:v>
       </x:c>
       <x:c r="E12" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F12" s="10" t="n">
         <x:f>D12</x:f>
-        <x:v>13269.37</x:v>
+        <x:v>20140.4</x:v>
       </x:c>
       <x:c r="G12" s="10" t="n">
         <x:f>F12*(1+E12)</x:f>
-        <x:v>15923.244</x:v>
+        <x:v>24168.48</x:v>
       </x:c>
       <x:c r="H12" s="19" t="str">
-        <x:v>https://trainingshowroom.com/maszyny-silowe/2939-maszyna-do-przysiadow-proud-champion.html</x:v>
+        <x:v>https://trainingshowroom.com/maszyny-silowe/2992-maszyna-leverage-chest-press-proud-champion.html</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="6" t="str">
-        <x:v>Maszyny na nogi</x:v>
+        <x:v>Maszyny na plecy</x:v>
       </x:c>
       <x:c r="B13" s="19" t="str">
-        <x:v>Seated Leg Extension Plate Loaded PROUD Champion</x:v>
+        <x:v>Ławka do wiosłowania PROUD Champion</x:v>
       </x:c>
       <x:c r="C13" s="6" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D13" s="10" t="n">
-        <x:v>11108.99</x:v>
+        <x:v>8169.88</x:v>
       </x:c>
       <x:c r="E13" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F13" s="10" t="n">
         <x:f>D13</x:f>
-        <x:v>11108.99</x:v>
+        <x:v>8169.88</x:v>
       </x:c>
       <x:c r="G13" s="10" t="n">
         <x:f>F13*(1+E13)</x:f>
-        <x:v>13330.787999999999</x:v>
+        <x:v>9803.856</x:v>
       </x:c>
       <x:c r="H13" s="19" t="str">
-        <x:v>https://trainingshowroom.com/maszyny-na-wolny-ciezar/3404-maszyna-seated-leg-extension-plate-loaded-proud-champion.html</x:v>
+        <x:v>https://trainingshowroom.com/lawki-treningowe/2946-lawka-do-wioslowania-proud-champion.html</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1018,223 +1039,223 @@
         <x:v>Maszyny na nogi</x:v>
       </x:c>
       <x:c r="B14" s="19" t="str">
-        <x:v>Maszyna do treningu łydek PROUD Champion</x:v>
+        <x:v>Maszyna do przysiadów Hack PROUD Champion</x:v>
       </x:c>
       <x:c r="C14" s="6" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D14" s="10" t="n">
-        <x:v>6284.21</x:v>
+        <x:v>13269.37</x:v>
       </x:c>
       <x:c r="E14" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F14" s="10" t="n">
         <x:f>D14</x:f>
-        <x:v>6284.21</x:v>
+        <x:v>13269.37</x:v>
       </x:c>
       <x:c r="G14" s="10" t="n">
         <x:f>F14*(1+E14)</x:f>
-        <x:v>7541.052</x:v>
+        <x:v>15923.244</x:v>
       </x:c>
       <x:c r="H14" s="19" t="str">
-        <x:v>https://trainingshowroom.com/maszyny-silowe/2938-maszyna-do-lydek-proud-champion.html</x:v>
+        <x:v>https://trainingshowroom.com/maszyny-silowe/2939-maszyna-do-przysiadow-proud-champion.html</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="6" t="str">
-        <x:v>Ławki i gryfy</x:v>
+        <x:v>Maszyny na nogi</x:v>
       </x:c>
       <x:c r="B15" s="19" t="str">
-        <x:v>Modlitewnik PROUD Champion</x:v>
+        <x:v>Seated Leg Extension Plate Loaded PROUD Champion</x:v>
       </x:c>
       <x:c r="C15" s="6" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D15" s="10" t="n">
-        <x:v>4502.57</x:v>
+        <x:v>11108.99</x:v>
       </x:c>
       <x:c r="E15" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F15" s="10" t="n">
         <x:f>D15</x:f>
-        <x:v>4502.57</x:v>
+        <x:v>11108.99</x:v>
       </x:c>
       <x:c r="G15" s="10" t="n">
         <x:f>F15*(1+E15)</x:f>
-        <x:v>5403.084</x:v>
+        <x:v>13330.787999999999</x:v>
       </x:c>
       <x:c r="H15" s="19" t="str">
-        <x:v>https://trainingshowroom.com/champion/2970-modlitewnik-proud-champion.html?search_query=Modlitewnik</x:v>
+        <x:v>https://trainingshowroom.com/maszyny-na-wolny-ciezar/3404-maszyna-seated-leg-extension-plate-loaded-proud-champion.html</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="6" t="str">
-        <x:v>Ławki i gryfy</x:v>
+        <x:v>Maszyny na nogi</x:v>
       </x:c>
       <x:c r="B16" s="19" t="str">
-        <x:v>Gryf olimpijski treningowy łamany Curl Silver PROUD</x:v>
+        <x:v>Maszyna do treningu łydek PROUD Champion</x:v>
       </x:c>
       <x:c r="C16" s="6" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D16" s="10" t="n">
-        <x:v>499.99</x:v>
+        <x:v>6284.21</x:v>
       </x:c>
       <x:c r="E16" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F16" s="10" t="n">
         <x:f>D16</x:f>
-        <x:v>499.99</x:v>
+        <x:v>6284.21</x:v>
       </x:c>
       <x:c r="G16" s="10" t="n">
         <x:f>F16*(1+E16)</x:f>
-        <x:v>599.9879999999999</x:v>
+        <x:v>7541.052</x:v>
       </x:c>
       <x:c r="H16" s="19" t="str">
-        <x:v>https://trainingshowroom.com/sztangi/2596-gryf-olimpijski-treningowy-lamany-silver-proud.html</x:v>
+        <x:v>https://trainingshowroom.com/maszyny-silowe/2938-maszyna-do-lydek-proud-champion.html</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="6" t="str">
-        <x:v>Hantle</x:v>
+        <x:v>Ławki i gryfy</x:v>
       </x:c>
       <x:c r="B17" s="19" t="str">
-        <x:v>Hantle poliuretanowe Studio PROUD, zestaw 1-10 kg</x:v>
+        <x:v>Modlitewnik PROUD Champion</x:v>
       </x:c>
       <x:c r="C17" s="6" t="str">
-        <x:v>2 zestawy</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D17" s="10" t="n">
-        <x:v>8241.58</x:v>
+        <x:v>4502.57</x:v>
       </x:c>
       <x:c r="E17" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F17" s="10" t="n">
         <x:f>D17</x:f>
-        <x:v>8241.58</x:v>
+        <x:v>4502.57</x:v>
       </x:c>
       <x:c r="G17" s="10" t="n">
         <x:f>F17*(1+E17)</x:f>
-        <x:v>9889.895999999999</x:v>
+        <x:v>5403.084</x:v>
       </x:c>
       <x:c r="H17" s="19" t="str">
-        <x:v>https://trainingshowroom.com/hantle-i-kettlebells/3467-hantle-poliuretanowe-studio-zestaw-proud.html</x:v>
+        <x:v>https://trainingshowroom.com/champion/2970-modlitewnik-proud-champion.html?search_query=Modlitewnik</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="6" t="str">
-        <x:v>Cardio</x:v>
+        <x:v>Ławki i gryfy</x:v>
       </x:c>
       <x:c r="B18" s="19" t="str">
-        <x:v>Ergometr wioślarski AIR 2.0 PROUD</x:v>
+        <x:v>Gryf olimpijski treningowy łamany Curl Silver PROUD</x:v>
       </x:c>
       <x:c r="C18" s="6" t="str">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D18" s="10" t="n">
-        <x:v>10720.12</x:v>
+        <x:v>499.99</x:v>
       </x:c>
       <x:c r="E18" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F18" s="10" t="n">
         <x:f>D18</x:f>
-        <x:v>10720.12</x:v>
+        <x:v>499.99</x:v>
       </x:c>
       <x:c r="G18" s="10" t="n">
         <x:f>F18*(1+E18)</x:f>
-        <x:v>12864.144</x:v>
+        <x:v>599.9879999999999</x:v>
       </x:c>
       <x:c r="H18" s="19" t="str">
-        <x:v>https://trainingshowroom.com/ergometry/2782-ergometr-wioslarski-air-proud-20.html?hsCtaAttrib=186811937891</x:v>
+        <x:v>https://trainingshowroom.com/sztangi/2596-gryf-olimpijski-treningowy-lamany-silver-proud.html</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="6" t="str">
-        <x:v>Cardio</x:v>
+        <x:v>Hantle</x:v>
       </x:c>
       <x:c r="B19" s="19" t="str">
-        <x:v>Air Runner, bieżnia treningowa 2.0 Elite PROUD Outlet</x:v>
+        <x:v>Hantle poliuretanowe Studio PROUD, zestaw 1-10 kg</x:v>
       </x:c>
       <x:c r="C19" s="6" t="str">
-        <x:v>1</x:v>
+        <x:v>2 zestawy</x:v>
       </x:c>
       <x:c r="D19" s="10" t="n">
-        <x:v>16905.12</x:v>
+        <x:v>8241.58</x:v>
       </x:c>
       <x:c r="E19" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F19" s="10" t="n">
         <x:f>D19</x:f>
-        <x:v>16905.12</x:v>
+        <x:v>8241.58</x:v>
       </x:c>
       <x:c r="G19" s="10" t="n">
         <x:f>F19*(1+E19)</x:f>
-        <x:v>20286.143999999997</x:v>
+        <x:v>9889.895999999999</x:v>
       </x:c>
       <x:c r="H19" s="19" t="str">
-        <x:v>https://trainingshowroom.com/bieznie/3501-air-runner-bieznia-treningowa-20-elite-proud-outlet.html</x:v>
+        <x:v>https://trainingshowroom.com/hantle-i-kettlebells/3467-hantle-poliuretanowe-studio-zestaw-proud.html</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="6" t="str">
-        <x:v>Drabinki i drobny sprzęt</x:v>
+        <x:v>Cardio</x:v>
       </x:c>
       <x:c r="B20" s="19" t="str">
-        <x:v>Poręcze do drabinki PROUD Champion Outlet</x:v>
+        <x:v>Ergometr wioślarski AIR 2.0 PROUD</x:v>
       </x:c>
       <x:c r="C20" s="6" t="str">
         <x:v>2</x:v>
       </x:c>
       <x:c r="D20" s="10" t="n">
-        <x:v>2451.86</x:v>
+        <x:v>10720.12</x:v>
       </x:c>
       <x:c r="E20" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F20" s="10" t="n">
         <x:f>D20</x:f>
-        <x:v>2451.86</x:v>
+        <x:v>10720.12</x:v>
       </x:c>
       <x:c r="G20" s="10" t="n">
         <x:f>F20*(1+E20)</x:f>
-        <x:v>2942.232</x:v>
+        <x:v>12864.144</x:v>
       </x:c>
       <x:c r="H20" s="19" t="str">
-        <x:v>https://trainingshowroom.com/outlet/3584-porecze-do-drabinki-proud-champion-outlet.html</x:v>
+        <x:v>https://trainingshowroom.com/ergometry/2782-ergometr-wioslarski-air-proud-20.html?hsCtaAttrib=186811937891</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="6" t="str">
-        <x:v>Drabinki i drobny sprzęt</x:v>
+        <x:v>Cardio</x:v>
       </x:c>
       <x:c r="B21" s="19" t="str">
-        <x:v>Drabinka gimnastyczna PROUD</x:v>
+        <x:v>Air Runner, bieżnia treningowa 2.0 Elite PROUD Outlet</x:v>
       </x:c>
       <x:c r="C21" s="6" t="str">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D21" s="10" t="n">
-        <x:v>1939.18</x:v>
+        <x:v>16905.12</x:v>
       </x:c>
       <x:c r="E21" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F21" s="10" t="n">
         <x:f>D21</x:f>
-        <x:v>1939.18</x:v>
+        <x:v>16905.12</x:v>
       </x:c>
       <x:c r="G21" s="10" t="n">
         <x:f>F21*(1+E21)</x:f>
-        <x:v>2327.016</x:v>
+        <x:v>20286.143999999997</x:v>
       </x:c>
       <x:c r="H21" s="19" t="str">
-        <x:v>https://trainingshowroom.com/sprzet-gimnastyczny/2272-drabinka-gimnastyczna-proud.html</x:v>
+        <x:v>https://trainingshowroom.com/bieznie/3501-air-runner-bieznia-treningowa-20-elite-proud-outlet.html</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -1242,27 +1263,27 @@
         <x:v>Drabinki i drobny sprzęt</x:v>
       </x:c>
       <x:c r="B22" s="19" t="str">
-        <x:v>Drążek do podciągania do drabinki PROUD Champion Outlet</x:v>
+        <x:v>Poręcze do drabinki PROUD Champion Outlet</x:v>
       </x:c>
       <x:c r="C22" s="6" t="str">
         <x:v>2</x:v>
       </x:c>
       <x:c r="D22" s="10" t="n">
-        <x:v>1251.38</x:v>
+        <x:v>2451.86</x:v>
       </x:c>
       <x:c r="E22" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F22" s="10" t="n">
         <x:f>D22</x:f>
-        <x:v>1251.38</x:v>
+        <x:v>2451.86</x:v>
       </x:c>
       <x:c r="G22" s="10" t="n">
         <x:f>F22*(1+E22)</x:f>
-        <x:v>1501.6560000000002</x:v>
+        <x:v>2942.232</x:v>
       </x:c>
       <x:c r="H22" s="19" t="str">
-        <x:v>https://trainingshowroom.com/outlet/3585-drazek-do-podciagania-do-drabinki-proud-champion-outlet.html</x:v>
+        <x:v>https://trainingshowroom.com/outlet/3584-porecze-do-drabinki-proud-champion-outlet.html</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -1270,172 +1291,396 @@
         <x:v>Drabinki i drobny sprzęt</x:v>
       </x:c>
       <x:c r="B23" s="19" t="str">
-        <x:v>Podkładki do przysiadów PROUD</x:v>
+        <x:v>Drabinka gimnastyczna PROUD</x:v>
       </x:c>
       <x:c r="C23" s="6" t="str">
-        <x:v>1 komplet</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D23" s="10" t="n">
-        <x:v>79.99</x:v>
+        <x:v>1939.18</x:v>
       </x:c>
       <x:c r="E23" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F23" s="10" t="n">
         <x:f>D23</x:f>
-        <x:v>79.99</x:v>
+        <x:v>1939.18</x:v>
       </x:c>
       <x:c r="G23" s="10" t="n">
         <x:f>F23*(1+E23)</x:f>
-        <x:v>95.98799999999999</x:v>
+        <x:v>2327.016</x:v>
       </x:c>
       <x:c r="H23" s="19" t="str">
-        <x:v>https://trainingshowroom.com/gumy-i-rollery/3356-podkladki-do-przysiadow-proud.html</x:v>
+        <x:v>https://trainingshowroom.com/sprzet-gimnastyczny/2272-drabinka-gimnastyczna-proud.html</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="6" t="str">
-        <x:v>Opcjonalne uzupełnienie</x:v>
+        <x:v>Drabinki i drobny sprzęt</x:v>
       </x:c>
       <x:c r="B24" s="19" t="str">
-        <x:v>Kettlebell żeliwny PRO, zestaw PROUD</x:v>
+        <x:v>Drążek do podciągania do drabinki PROUD Champion Outlet</x:v>
       </x:c>
       <x:c r="C24" s="6" t="str">
-        <x:v>1 zestaw</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D24" s="10" t="n">
-        <x:v>2625.99</x:v>
+        <x:v>1251.38</x:v>
       </x:c>
       <x:c r="E24" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F24" s="10" t="n">
         <x:f>D24</x:f>
-        <x:v>2625.99</x:v>
+        <x:v>1251.38</x:v>
       </x:c>
       <x:c r="G24" s="10" t="n">
         <x:f>F24*(1+E24)</x:f>
-        <x:v>3151.1879999999996</x:v>
+        <x:v>1501.6560000000002</x:v>
       </x:c>
       <x:c r="H24" s="19" t="str">
-        <x:v>https://trainingshowroom.com/hantle-i-kettlebells/3465-hantla-proud-kettlebell-zestaw.html</x:v>
+        <x:v>https://trainingshowroom.com/outlet/3585-drazek-do-podciagania-do-drabinki-proud-champion-outlet.html</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="6" t="str">
-        <x:v>Opcjonalne uzupełnienie</x:v>
+        <x:v>Drabinki i drobny sprzęt</x:v>
       </x:c>
       <x:c r="B25" s="19" t="str">
-        <x:v>Podłoga gumowa Standard PROUD pod kettlebell</x:v>
+        <x:v>Podkładki do przysiadów PROUD</x:v>
       </x:c>
       <x:c r="C25" s="6" t="str">
-        <x:v>4 szt.</x:v>
+        <x:v>1 komplet</x:v>
       </x:c>
       <x:c r="D25" s="10" t="n">
-        <x:v>379.96</x:v>
+        <x:v>79.99</x:v>
       </x:c>
       <x:c r="E25" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F25" s="10" t="n">
         <x:f>D25</x:f>
-        <x:v>379.96</x:v>
+        <x:v>79.99</x:v>
       </x:c>
       <x:c r="G25" s="10" t="n">
         <x:f>F25*(1+E25)</x:f>
-        <x:v>455.95199999999994</x:v>
+        <x:v>95.98799999999999</x:v>
       </x:c>
       <x:c r="H25" s="19" t="str">
-        <x:v>https://trainingshowroom.com/podlogi/3427-podloga-gumowa-standard-proud.html</x:v>
+        <x:v>https://trainingshowroom.com/gumy-i-rollery/3356-podkladki-do-przysiadow-proud.html</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="6" t="str">
-        <x:v>Wyposażenie AV</x:v>
+        <x:v>Opcjonalne uzupełnienie</x:v>
       </x:c>
       <x:c r="B26" s="19" t="str">
-        <x:v>Projektor Full HD Epson EB-FH52</x:v>
+        <x:v>Kettlebell żeliwny PRO, zestaw PROUD</x:v>
       </x:c>
       <x:c r="C26" s="6" t="str">
-        <x:v>1</x:v>
+        <x:v>1 zestaw</x:v>
       </x:c>
       <x:c r="D26" s="10" t="n">
-        <x:v>4559</x:v>
+        <x:v>2625.99</x:v>
       </x:c>
       <x:c r="E26" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F26" s="10" t="n">
         <x:f>D26</x:f>
-        <x:v>4559</x:v>
+        <x:v>2625.99</x:v>
       </x:c>
       <x:c r="G26" s="10" t="n">
         <x:f>F26*(1+E26)</x:f>
-        <x:v>5470.8</x:v>
+        <x:v>3151.1879999999996</x:v>
       </x:c>
       <x:c r="H26" s="19" t="str">
-        <x:v>https://www.x-kom.pl/p/1224184-projektor-epson-eb-fh52.html</x:v>
+        <x:v>https://trainingshowroom.com/hantle-i-kettlebells/3465-hantla-proud-kettlebell-zestaw.html</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="6" t="str">
-        <x:v>Wyposażenie AV</x:v>
+        <x:v>Opcjonalne uzupełnienie</x:v>
       </x:c>
       <x:c r="B27" s="19" t="str">
-        <x:v>Mobilny zestaw audio LD Systems Roadbuddy 10 HHD 2</x:v>
+        <x:v>Podłoga gumowa Standard PROUD pod kettlebell</x:v>
       </x:c>
       <x:c r="C27" s="6" t="str">
-        <x:v>1</x:v>
+        <x:v>4 szt.</x:v>
       </x:c>
       <x:c r="D27" s="10" t="n">
-        <x:v>3507</x:v>
+        <x:v>379.96</x:v>
       </x:c>
       <x:c r="E27" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F27" s="10" t="n">
         <x:f>D27</x:f>
-        <x:v>3507</x:v>
+        <x:v>379.96</x:v>
       </x:c>
       <x:c r="G27" s="10" t="n">
         <x:f>F27*(1+E27)</x:f>
-        <x:v>4208.4</x:v>
+        <x:v>455.95199999999994</x:v>
       </x:c>
       <x:c r="H27" s="19" t="str">
-        <x:v>https://www.ceneo.pl/89383056</x:v>
+        <x:v>https://trainingshowroom.com/podlogi/3427-podloga-gumowa-standard-proud.html</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="6"/>
-      <x:c r="B28" s="6"/>
-      <x:c r="C28" s="6"/>
-      <x:c r="D28" s="10"/>
-      <x:c r="E28" s="6"/>
-      <x:c r="F28" s="10"/>
-      <x:c r="G28" s="10"/>
-      <x:c r="H28" s="6"/>
+      <x:c r="A28" s="6" t="str">
+        <x:v>Wyposażenie AV</x:v>
+      </x:c>
+      <x:c r="B28" s="19" t="str">
+        <x:v>Lustra na jedną ścianę pomieszczenia</x:v>
+      </x:c>
+      <x:c r="C28" s="6" t="str">
+        <x:v>ok. 16 m²</x:v>
+      </x:c>
+      <x:c r="D28" s="10" t="n">
+        <x:v>6500</x:v>
+      </x:c>
+      <x:c r="E28" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F28" s="10" t="n">
+        <x:f>D28</x:f>
+        <x:v>6500</x:v>
+      </x:c>
+      <x:c r="G28" s="10" t="n">
+        <x:f>F28*(1+E28)</x:f>
+        <x:v>7800</x:v>
+      </x:c>
+      <x:c r="H28" s="19" t="str">
+        <x:v>Cena orientacyjna, jedna pełna ściana</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="17" t="str">
+      <x:c r="A29" s="6" t="str">
+        <x:v>Wyposażenie AV</x:v>
+      </x:c>
+      <x:c r="B29" s="19" t="str">
+        <x:v>Projektor Full HD Epson EB-FH52</x:v>
+      </x:c>
+      <x:c r="C29" s="6" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D29" s="10" t="n">
+        <x:v>4559</x:v>
+      </x:c>
+      <x:c r="E29" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F29" s="10" t="n">
+        <x:f>D29</x:f>
+        <x:v>4559</x:v>
+      </x:c>
+      <x:c r="G29" s="10" t="n">
+        <x:f>F29*(1+E29)</x:f>
+        <x:v>5470.8</x:v>
+      </x:c>
+      <x:c r="H29" s="19" t="str">
+        <x:v>https://www.x-kom.pl/p/1224184-projektor-epson-eb-fh52.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="6" t="str">
+        <x:v>Wyposażenie AV</x:v>
+      </x:c>
+      <x:c r="B30" s="19" t="str">
+        <x:v>Ekran projekcyjny ręczny Avtek Cinema 280</x:v>
+      </x:c>
+      <x:c r="C30" s="6" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D30" s="10" t="n">
+        <x:v>739</x:v>
+      </x:c>
+      <x:c r="E30" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F30" s="10" t="n">
+        <x:f>D30</x:f>
+        <x:v>739</x:v>
+      </x:c>
+      <x:c r="G30" s="10" t="n">
+        <x:f>F30*(1+E30)</x:f>
+        <x:v>886.8</x:v>
+      </x:c>
+      <x:c r="H30" s="19" t="str">
+        <x:v>https://www.al.to/p/537648-ekran-projekcyjny-avtek-ekran-projekcyjny-cinema-280.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="6" t="str">
+        <x:v>Wyposażenie AV</x:v>
+      </x:c>
+      <x:c r="B31" s="19" t="str">
+        <x:v>Kabel HDMI światłowodowy 20 m Claroc</x:v>
+      </x:c>
+      <x:c r="C31" s="6" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D31" s="10" t="n">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="E31" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F31" s="10" t="n">
+        <x:f>D31</x:f>
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="G31" s="10" t="n">
+        <x:f>F31*(1+E31)</x:f>
+        <x:v>250.79999999999998</x:v>
+      </x:c>
+      <x:c r="H31" s="19" t="str">
+        <x:v>https://www.x-kom.pl/p/1277224-kabel-hdmi-claroc-optyczny-hdmi-21-8k-120hz-20m.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="6" t="str">
+        <x:v>Wyposażenie AV</x:v>
+      </x:c>
+      <x:c r="B32" s="19" t="str">
+        <x:v>Zestaw stereo Bluetooth Triangle AIO TWIN</x:v>
+      </x:c>
+      <x:c r="C32" s="6" t="str">
+        <x:v>1 komplet</x:v>
+      </x:c>
+      <x:c r="D32" s="10" t="n">
+        <x:v>2990</x:v>
+      </x:c>
+      <x:c r="E32" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F32" s="10" t="n">
+        <x:f>D32</x:f>
+        <x:v>2990</x:v>
+      </x:c>
+      <x:c r="G32" s="10" t="n">
+        <x:f>F32*(1+E32)</x:f>
+        <x:v>3588</x:v>
+      </x:c>
+      <x:c r="H32" s="19" t="str">
+        <x:v>https://avstore.pl/monitory-aktywne/triangle-aio-twin-aktywne-kolumny-podstawkowe-z-bluetooth-wi-fi.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="6" t="str">
+        <x:v>Wyposażenie AV</x:v>
+      </x:c>
+      <x:c r="B33" s="19" t="str">
+        <x:v>Zestaw mikrofonowy nagłowny Tonsil ZP 12</x:v>
+      </x:c>
+      <x:c r="C33" s="6" t="str">
+        <x:v>1 komplet</x:v>
+      </x:c>
+      <x:c r="D33" s="10" t="n">
+        <x:v>1699</x:v>
+      </x:c>
+      <x:c r="E33" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F33" s="10" t="n">
+        <x:f>D33</x:f>
+        <x:v>1699</x:v>
+      </x:c>
+      <x:c r="G33" s="10" t="n">
+        <x:f>F33*(1+E33)</x:f>
+        <x:v>2038.8</x:v>
+      </x:c>
+      <x:c r="H33" s="19" t="str">
+        <x:v>https://avstore.pl/naglosnienie-przenosne/zestaw-tonsil-zp-12-przenosny-bezprzewodowy-system-naglosnieniowy-pa-mikrofon-uhf-mikrofon-naglowny-statyw-m502-102.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="6" t="str">
+        <x:v>Wyposażenie AV</x:v>
+      </x:c>
+      <x:c r="B34" s="19" t="str">
+        <x:v>Uchwyty ścienne do głośników Gravity SP WMBS 30 B</x:v>
+      </x:c>
+      <x:c r="C34" s="6" t="str">
+        <x:v>2 szt.</x:v>
+      </x:c>
+      <x:c r="D34" s="10" t="n">
+        <x:v>319.98</x:v>
+      </x:c>
+      <x:c r="E34" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F34" s="10" t="n">
+        <x:f>D34</x:f>
+        <x:v>319.98</x:v>
+      </x:c>
+      <x:c r="G34" s="10" t="n">
+        <x:f>F34*(1+E34)</x:f>
+        <x:v>383.976</x:v>
+      </x:c>
+      <x:c r="H34" s="19" t="str">
+        <x:v>https://www.ablosklep.com/gravity-sp-wmbs-30-b-wychylny-obrotowy-uchwyt-scienny-do-glosnikow-do-30-kg-czarny-p-3991.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="6" t="str">
+        <x:v>Wyposażenie AV</x:v>
+      </x:c>
+      <x:c r="B35" s="19" t="str">
+        <x:v>Kabel audio mini jack 3,5 mm - 2x RCA 10 m Lindy</x:v>
+      </x:c>
+      <x:c r="C35" s="6" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D35" s="10" t="n">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="E35" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F35" s="10" t="n">
+        <x:f>D35</x:f>
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="G35" s="10" t="n">
+        <x:f>F35*(1+E35)</x:f>
+        <x:v>80.39999999999999</x:v>
+      </x:c>
+      <x:c r="H35" s="19" t="str">
+        <x:v>https://sklep.rms.pl/lindy-35337-kabel-mini-jack-3-5mm-2x-rca-cromo-line-10m</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="6"/>
+      <x:c r="B36" s="6"/>
+      <x:c r="C36" s="6"/>
+      <x:c r="D36" s="10"/>
+      <x:c r="E36" s="6"/>
+      <x:c r="F36" s="10"/>
+      <x:c r="G36" s="10"/>
+      <x:c r="H36" s="6"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="17" t="str">
         <x:v>Razem</x:v>
       </x:c>
-      <x:c r="B29" s="17"/>
-      <x:c r="C29" s="17"/>
-      <x:c r="D29" s="18"/>
-      <x:c r="E29" s="17"/>
-      <x:c r="F29" s="18" t="n">
-        <x:f>SUM(F2:F27)</x:f>
-        <x:v>154627.97999999995</x:v>
-      </x:c>
-      <x:c r="G29" s="18" t="n">
-        <x:f>SUM(G2:G27)</x:f>
-        <x:v>185553.57599999994</x:v>
-      </x:c>
-      <x:c r="H29" s="17"/>
+      <x:c r="B37" s="17"/>
+      <x:c r="C37" s="17"/>
+      <x:c r="D37" s="18"/>
+      <x:c r="E37" s="17"/>
+      <x:c r="F37" s="18" t="n">
+        <x:f>SUM(F2:F35)</x:f>
+        <x:v>191955.24</x:v>
+      </x:c>
+      <x:c r="G37" s="18" t="n">
+        <x:f>SUM(G2:G35)</x:f>
+        <x:v>230346.2879999999</x:v>
+      </x:c>
+      <x:c r="H37" s="17"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A29:C29"/>
+    <x:mergeCell ref="A37:C37"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Update kettlebell mat quantity
</commit_message>
<xml_diff>
--- a/outputs/wyposazenie-silowni/wyposazenie-silowni-zsz5-2027.xlsx
+++ b/outputs/wyposazenie-silowni/wyposazenie-silowni-zsz5-2027.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Podsumowanie" sheetId="1" r:id="Rbc6db7a558bb4d08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kosztorys siłowni" sheetId="2" r:id="R51aa0fdbf3c94daf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Podsumowanie" sheetId="1" r:id="R4a0f100a88fa4894"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kosztorys siłowni" sheetId="2" r:id="R22f13cdcf04e407d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -365,7 +365,7 @@
       </x:c>
       <x:c r="B6" s="10" t="n">
         <x:f>'Kosztorys siłowni'!F37</x:f>
-        <x:v>191955.24</x:v>
+        <x:v>192415.21</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -374,7 +374,7 @@
       </x:c>
       <x:c r="B7" s="12" t="n">
         <x:f>'Kosztorys siłowni'!G37</x:f>
-        <x:v>230346.2879999999</x:v>
+        <x:v>230898.25199999992</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -414,7 +414,7 @@
       </x:c>
       <x:c r="E11" s="15" t="n">
         <x:f>D11/$B$7</x:f>
-        <x:v>0.08490000064598395</x:v>
+        <x:v>0.08469704655884534</x:v>
       </x:c>
       <x:c r="F11" s="6" t="str"/>
     </x:row>
@@ -435,7 +435,7 @@
       </x:c>
       <x:c r="E12" s="15" t="n">
         <x:f>D12/$B$7</x:f>
-        <x:v>0.06445565122369154</x:v>
+        <x:v>0.06430156950690126</x:v>
       </x:c>
       <x:c r="F12" s="6" t="str"/>
     </x:row>
@@ -456,7 +456,7 @@
       </x:c>
       <x:c r="E13" s="15" t="n">
         <x:f>D13/$B$7</x:f>
-        <x:v>0.004799608492063047</x:v>
+        <x:v>0.004788134992031037</x:v>
       </x:c>
       <x:c r="F13" s="6" t="str"/>
     </x:row>
@@ -477,7 +477,7 @@
       </x:c>
       <x:c r="E14" s="15" t="n">
         <x:f>D14/$B$7</x:f>
-        <x:v>0.29616883602656546</x:v>
+        <x:v>0.29546084220680896</x:v>
       </x:c>
       <x:c r="F14" s="6" t="str"/>
     </x:row>
@@ -498,7 +498,7 @@
       </x:c>
       <x:c r="E15" s="15" t="n">
         <x:f>D15/$B$7</x:f>
-        <x:v>0.042561380455151954</x:v>
+        <x:v>0.04245963715654289</x:v>
       </x:c>
       <x:c r="F15" s="6" t="str"/>
     </x:row>
@@ -519,7 +519,7 @@
       </x:c>
       <x:c r="E16" s="15" t="n">
         <x:f>D16/$B$7</x:f>
-        <x:v>0.15973812436690976</x:v>
+        <x:v>0.15935626918474902</x:v>
       </x:c>
       <x:c r="F16" s="6" t="str"/>
     </x:row>
@@ -540,7 +540,7 @@
       </x:c>
       <x:c r="E17" s="15" t="n">
         <x:f>D17/$B$7</x:f>
-        <x:v>0.0260610754882232</x:v>
+        <x:v>0.02599877629216527</x:v>
       </x:c>
       <x:c r="F17" s="6" t="str"/>
     </x:row>
@@ -561,7 +561,7 @@
       </x:c>
       <x:c r="E18" s="15" t="n">
         <x:f>D18/$B$7</x:f>
-        <x:v>0.04293490503306918</x:v>
+        <x:v>0.04283226882116025</x:v>
       </x:c>
       <x:c r="F18" s="6" t="str"/>
     </x:row>
@@ -582,7 +582,7 @@
       </x:c>
       <x:c r="E19" s="15" t="n">
         <x:f>D19/$B$7</x:f>
-        <x:v>0.14391500851969455</x:v>
+        <x:v>0.14357097861442455</x:v>
       </x:c>
       <x:c r="F19" s="6" t="str"/>
     </x:row>
@@ -603,7 +603,7 @@
       </x:c>
       <x:c r="E20" s="15" t="n">
         <x:f>D20/$B$7</x:f>
-        <x:v>0.029811168478651597</x:v>
+        <x:v>0.029739904657225393</x:v>
       </x:c>
       <x:c r="F20" s="6" t="str"/>
     </x:row>
@@ -616,15 +616,15 @@
       </x:c>
       <x:c r="C21" s="10" t="n">
         <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A21)</x:f>
-        <x:v>3005.95</x:v>
+        <x:v>3465.9199999999996</x:v>
       </x:c>
       <x:c r="D21" s="10" t="n">
         <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A21)</x:f>
-        <x:v>3607.1399999999994</x:v>
+        <x:v>4159.103999999999</x:v>
       </x:c>
       <x:c r="E21" s="15" t="n">
         <x:f>D21/$B$7</x:f>
-        <x:v>0.01565964023696358</x:v>
+        <x:v>0.01801271323613139</x:v>
       </x:c>
       <x:c r="F21" s="6" t="str"/>
     </x:row>
@@ -645,7 +645,7 @@
       </x:c>
       <x:c r="E22" s="15" t="n">
         <x:f>D22/$B$7</x:f>
-        <x:v>0.08899460103303251</x:v>
+        <x:v>0.0887818587730149</x:v>
       </x:c>
       <x:c r="F22" s="6" t="str"/>
     </x:row>
@@ -1403,24 +1403,24 @@
         <x:v>Opcjonalne uzupełnienie</x:v>
       </x:c>
       <x:c r="B27" s="19" t="str">
-        <x:v>Podłoga gumowa Standard PROUD pod kettlebell</x:v>
+        <x:v>Podłoga gumowa Standard PROUD 15 mm pod kettlebell</x:v>
       </x:c>
       <x:c r="C27" s="6" t="str">
-        <x:v>4 szt.</x:v>
+        <x:v>7 szt.</x:v>
       </x:c>
       <x:c r="D27" s="10" t="n">
-        <x:v>379.96</x:v>
+        <x:v>839.93</x:v>
       </x:c>
       <x:c r="E27" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F27" s="10" t="n">
         <x:f>D27</x:f>
-        <x:v>379.96</x:v>
+        <x:v>839.93</x:v>
       </x:c>
       <x:c r="G27" s="10" t="n">
         <x:f>F27*(1+E27)</x:f>
-        <x:v>455.95199999999994</x:v>
+        <x:v>1007.9159999999999</x:v>
       </x:c>
       <x:c r="H27" s="19" t="str">
         <x:v>https://trainingshowroom.com/podlogi/3427-podloga-gumowa-standard-proud.html</x:v>
@@ -1670,11 +1670,11 @@
       <x:c r="E37" s="17"/>
       <x:c r="F37" s="18" t="n">
         <x:f>SUM(F2:F35)</x:f>
-        <x:v>191955.24</x:v>
+        <x:v>192415.21</x:v>
       </x:c>
       <x:c r="G37" s="18" t="n">
         <x:f>SUM(G2:G35)</x:f>
-        <x:v>230346.2879999999</x:v>
+        <x:v>230898.25199999992</x:v>
       </x:c>
       <x:c r="H37" s="17"/>
     </x:row>

</xml_diff>

<commit_message>
Update puzzle mats and projection screen
</commit_message>
<xml_diff>
--- a/outputs/wyposazenie-silowni/wyposazenie-silowni-zsz5-2027.xlsx
+++ b/outputs/wyposazenie-silowni/wyposazenie-silowni-zsz5-2027.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Podsumowanie" sheetId="1" r:id="R4a0f100a88fa4894"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kosztorys siłowni" sheetId="2" r:id="R22f13cdcf04e407d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Podsumowanie" sheetId="1" r:id="R108cd9d574c54b27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kosztorys siłowni" sheetId="2" r:id="R1577557e42424281"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -365,7 +365,7 @@
       </x:c>
       <x:c r="B6" s="10" t="n">
         <x:f>'Kosztorys siłowni'!F37</x:f>
-        <x:v>192415.21</x:v>
+        <x:v>193455.18</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -374,7 +374,7 @@
       </x:c>
       <x:c r="B7" s="12" t="n">
         <x:f>'Kosztorys siłowni'!G37</x:f>
-        <x:v>230898.25199999992</x:v>
+        <x:v>232146.21599999993</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -414,7 +414,7 @@
       </x:c>
       <x:c r="E11" s="15" t="n">
         <x:f>D11/$B$7</x:f>
-        <x:v>0.08469704655884534</x:v>
+        <x:v>0.08424173495897087</x:v>
       </x:c>
       <x:c r="F11" s="6" t="str"/>
     </x:row>
@@ -435,7 +435,7 @@
       </x:c>
       <x:c r="E12" s="15" t="n">
         <x:f>D12/$B$7</x:f>
-        <x:v>0.06430156950690126</x:v>
+        <x:v>0.06395589924239818</x:v>
       </x:c>
       <x:c r="F12" s="6" t="str"/>
     </x:row>
@@ -456,7 +456,7 @@
       </x:c>
       <x:c r="E13" s="15" t="n">
         <x:f>D13/$B$7</x:f>
-        <x:v>0.004788134992031037</x:v>
+        <x:v>0.004762395093271735</x:v>
       </x:c>
       <x:c r="F13" s="6" t="str"/>
     </x:row>
@@ -477,7 +477,7 @@
       </x:c>
       <x:c r="E14" s="15" t="n">
         <x:f>D14/$B$7</x:f>
-        <x:v>0.29546084220680896</x:v>
+        <x:v>0.2938725135196691</x:v>
       </x:c>
       <x:c r="F14" s="6" t="str"/>
     </x:row>
@@ -498,7 +498,7 @@
       </x:c>
       <x:c r="E15" s="15" t="n">
         <x:f>D15/$B$7</x:f>
-        <x:v>0.04245963715654289</x:v>
+        <x:v>0.042231384034276065</x:v>
       </x:c>
       <x:c r="F15" s="6" t="str"/>
     </x:row>
@@ -519,7 +519,7 @@
       </x:c>
       <x:c r="E16" s="15" t="n">
         <x:f>D16/$B$7</x:f>
-        <x:v>0.15935626918474902</x:v>
+        <x:v>0.15849960698907112</x:v>
       </x:c>
       <x:c r="F16" s="6" t="str"/>
     </x:row>
@@ -540,7 +540,7 @@
       </x:c>
       <x:c r="E17" s="15" t="n">
         <x:f>D17/$B$7</x:f>
-        <x:v>0.02599877629216527</x:v>
+        <x:v>0.025859012924854232</x:v>
       </x:c>
       <x:c r="F17" s="6" t="str"/>
     </x:row>
@@ -561,7 +561,7 @@
       </x:c>
       <x:c r="E18" s="15" t="n">
         <x:f>D18/$B$7</x:f>
-        <x:v>0.04283226882116025</x:v>
+        <x:v>0.04260201251783489</x:v>
       </x:c>
       <x:c r="F18" s="6" t="str"/>
     </x:row>
@@ -582,7 +582,7 @@
       </x:c>
       <x:c r="E19" s="15" t="n">
         <x:f>D19/$B$7</x:f>
-        <x:v>0.14357097861442455</x:v>
+        <x:v>0.14279917446511387</x:v>
       </x:c>
       <x:c r="F19" s="6" t="str"/>
     </x:row>
@@ -603,7 +603,7 @@
       </x:c>
       <x:c r="E20" s="15" t="n">
         <x:f>D20/$B$7</x:f>
-        <x:v>0.029739904657225393</x:v>
+        <x:v>0.02958002985497727</x:v>
       </x:c>
       <x:c r="F20" s="6" t="str"/>
     </x:row>
@@ -616,15 +616,15 @@
       </x:c>
       <x:c r="C21" s="10" t="n">
         <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A21)</x:f>
-        <x:v>3465.9199999999996</x:v>
+        <x:v>3825.89</x:v>
       </x:c>
       <x:c r="D21" s="10" t="n">
         <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A21)</x:f>
-        <x:v>4159.103999999999</x:v>
+        <x:v>4591.067999999999</x:v>
       </x:c>
       <x:c r="E21" s="15" t="n">
         <x:f>D21/$B$7</x:f>
-        <x:v>0.01801271323613139</x:v>
+        <x:v>0.019776622161267538</x:v>
       </x:c>
       <x:c r="F21" s="6" t="str"/>
     </x:row>
@@ -637,15 +637,15 @@
       </x:c>
       <x:c r="C22" s="10" t="n">
         <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A22)</x:f>
-        <x:v>17082.98</x:v>
+        <x:v>17762.98</x:v>
       </x:c>
       <x:c r="D22" s="10" t="n">
         <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A22)</x:f>
-        <x:v>20499.575999999997</x:v>
+        <x:v>21315.575999999997</x:v>
       </x:c>
       <x:c r="E22" s="15" t="n">
         <x:f>D22/$B$7</x:f>
-        <x:v>0.0887818587730149</x:v>
+        <x:v>0.09181961423829542</x:v>
       </x:c>
       <x:c r="F22" s="6" t="str"/>
     </x:row>
@@ -1406,21 +1406,21 @@
         <x:v>Podłoga gumowa Standard PROUD 15 mm pod kettlebell</x:v>
       </x:c>
       <x:c r="C27" s="6" t="str">
-        <x:v>7 szt.</x:v>
+        <x:v>10 szt.</x:v>
       </x:c>
       <x:c r="D27" s="10" t="n">
-        <x:v>839.93</x:v>
+        <x:v>1199.9</x:v>
       </x:c>
       <x:c r="E27" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F27" s="10" t="n">
         <x:f>D27</x:f>
-        <x:v>839.93</x:v>
+        <x:v>1199.9</x:v>
       </x:c>
       <x:c r="G27" s="10" t="n">
         <x:f>F27*(1+E27)</x:f>
-        <x:v>1007.9159999999999</x:v>
+        <x:v>1439.88</x:v>
       </x:c>
       <x:c r="H27" s="19" t="str">
         <x:v>https://trainingshowroom.com/podlogi/3427-podloga-gumowa-standard-proud.html</x:v>
@@ -1487,27 +1487,27 @@
         <x:v>Wyposażenie AV</x:v>
       </x:c>
       <x:c r="B30" s="19" t="str">
-        <x:v>Ekran projekcyjny ręczny Avtek Cinema 280</x:v>
+        <x:v>Ekran projekcyjny elektryczny Avtek Cinema Electric 300P</x:v>
       </x:c>
       <x:c r="C30" s="6" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D30" s="10" t="n">
-        <x:v>739</x:v>
+        <x:v>1419</x:v>
       </x:c>
       <x:c r="E30" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F30" s="10" t="n">
         <x:f>D30</x:f>
-        <x:v>739</x:v>
+        <x:v>1419</x:v>
       </x:c>
       <x:c r="G30" s="10" t="n">
         <x:f>F30*(1+E30)</x:f>
-        <x:v>886.8</x:v>
+        <x:v>1702.8</x:v>
       </x:c>
       <x:c r="H30" s="19" t="str">
-        <x:v>https://www.al.to/p/537648-ekran-projekcyjny-avtek-ekran-projekcyjny-cinema-280.html</x:v>
+        <x:v>https://www.x-kom.pl/p/711610-ekran-projekcyjny-avtek-ekran-elektryczny-cinema-electric-300p.html</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -1670,11 +1670,11 @@
       <x:c r="E37" s="17"/>
       <x:c r="F37" s="18" t="n">
         <x:f>SUM(F2:F35)</x:f>
-        <x:v>192415.21</x:v>
+        <x:v>193455.18</x:v>
       </x:c>
       <x:c r="G37" s="18" t="n">
         <x:f>SUM(G2:G35)</x:f>
-        <x:v>230898.25199999992</x:v>
+        <x:v>232146.21599999993</x:v>
       </x:c>
       <x:c r="H37" s="17"/>
     </x:row>

</xml_diff>

<commit_message>
Add functional training gym accessories
</commit_message>
<xml_diff>
--- a/outputs/wyposazenie-silowni/wyposazenie-silowni-zsz5-2027.xlsx
+++ b/outputs/wyposazenie-silowni/wyposazenie-silowni-zsz5-2027.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Podsumowanie" sheetId="1" r:id="R108cd9d574c54b27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kosztorys siłowni" sheetId="2" r:id="R1577557e42424281"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Podsumowanie" sheetId="1" r:id="Re94fda836aab4141"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kosztorys siłowni" sheetId="2" r:id="Ree162fc1c8804fd5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -348,7 +348,7 @@
         <x:v>Liczba pozycji</x:v>
       </x:c>
       <x:c r="B4" s="6" t="n">
-        <x:v>34</x:v>
+        <x:v>43</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -364,8 +364,8 @@
         <x:v>Suma cen sprzętu</x:v>
       </x:c>
       <x:c r="B6" s="10" t="n">
-        <x:f>'Kosztorys siłowni'!F37</x:f>
-        <x:v>193455.18</x:v>
+        <x:f>'Kosztorys siłowni'!F46</x:f>
+        <x:v>198904.63</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -373,8 +373,8 @@
         <x:v>Prognozowana suma +20%</x:v>
       </x:c>
       <x:c r="B7" s="12" t="n">
-        <x:f>'Kosztorys siłowni'!G37</x:f>
-        <x:v>232146.21599999993</x:v>
+        <x:f>'Kosztorys siłowni'!G46</x:f>
+        <x:v>238685.55599999992</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -405,16 +405,16 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A11)</x:f>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$44,'Kosztorys siłowni'!$A$2:$A$44,A11)</x:f>
         <x:v>16297</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A11)</x:f>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$44,'Kosztorys siłowni'!$A$2:$A$44,A11)</x:f>
         <x:v>19556.399999999998</x:v>
       </x:c>
       <x:c r="E11" s="15" t="n">
         <x:f>D11/$B$7</x:f>
-        <x:v>0.08424173495897087</x:v>
+        <x:v>0.08193373879733219</x:v>
       </x:c>
       <x:c r="F11" s="6" t="str"/>
     </x:row>
@@ -426,16 +426,16 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C12" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A12)</x:f>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$44,'Kosztorys siłowni'!$A$2:$A$44,A12)</x:f>
         <x:v>12372.6</x:v>
       </x:c>
       <x:c r="D12" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A12)</x:f>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$44,'Kosztorys siłowni'!$A$2:$A$44,A12)</x:f>
         <x:v>14847.119999999999</x:v>
       </x:c>
       <x:c r="E12" s="15" t="n">
         <x:f>D12/$B$7</x:f>
-        <x:v>0.06395589924239818</x:v>
+        <x:v>0.06220368022604603</x:v>
       </x:c>
       <x:c r="F12" s="6" t="str"/>
     </x:row>
@@ -447,16 +447,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C13" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A13)</x:f>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$44,'Kosztorys siłowni'!$A$2:$A$44,A13)</x:f>
         <x:v>921.31</x:v>
       </x:c>
       <x:c r="D13" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A13)</x:f>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$44,'Kosztorys siłowni'!$A$2:$A$44,A13)</x:f>
         <x:v>1105.572</x:v>
       </x:c>
       <x:c r="E13" s="15" t="n">
         <x:f>D13/$B$7</x:f>
-        <x:v>0.004762395093271735</x:v>
+        <x:v>0.004631918321861086</x:v>
       </x:c>
       <x:c r="F13" s="6" t="str"/>
     </x:row>
@@ -468,16 +468,16 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C14" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A14)</x:f>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$44,'Kosztorys siłowni'!$A$2:$A$44,A14)</x:f>
         <x:v>56851.16</x:v>
       </x:c>
       <x:c r="D14" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A14)</x:f>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$44,'Kosztorys siłowni'!$A$2:$A$44,A14)</x:f>
         <x:v>68221.39199999999</x:v>
       </x:c>
       <x:c r="E14" s="15" t="n">
         <x:f>D14/$B$7</x:f>
-        <x:v>0.2938725135196691</x:v>
+        <x:v>0.28582119983833465</x:v>
       </x:c>
       <x:c r="F14" s="6" t="str"/>
     </x:row>
@@ -489,16 +489,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C15" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A15)</x:f>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$44,'Kosztorys siłowni'!$A$2:$A$44,A15)</x:f>
         <x:v>8169.88</x:v>
       </x:c>
       <x:c r="D15" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A15)</x:f>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$44,'Kosztorys siłowni'!$A$2:$A$44,A15)</x:f>
         <x:v>9803.856</x:v>
       </x:c>
       <x:c r="E15" s="15" t="n">
         <x:f>D15/$B$7</x:f>
-        <x:v>0.042231384034276065</x:v>
+        <x:v>0.04107435809814986</x:v>
       </x:c>
       <x:c r="F15" s="6" t="str"/>
     </x:row>
@@ -510,16 +510,16 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C16" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A16)</x:f>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$44,'Kosztorys siłowni'!$A$2:$A$44,A16)</x:f>
         <x:v>30662.57</x:v>
       </x:c>
       <x:c r="D16" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A16)</x:f>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$44,'Kosztorys siłowni'!$A$2:$A$44,A16)</x:f>
         <x:v>36795.084</x:v>
       </x:c>
       <x:c r="E16" s="15" t="n">
         <x:f>D16/$B$7</x:f>
-        <x:v>0.15849960698907112</x:v>
+        <x:v>0.15415714556267499</x:v>
       </x:c>
       <x:c r="F16" s="6" t="str"/>
     </x:row>
@@ -528,19 +528,19 @@
         <x:v>Ławki i gryfy</x:v>
       </x:c>
       <x:c r="B17" s="6" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C17" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A17)</x:f>
-        <x:v>5002.5599999999995</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$44,'Kosztorys siłowni'!$A$2:$A$44,A17)</x:f>
+        <x:v>5802.549999999999</x:v>
       </x:c>
       <x:c r="D17" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A17)</x:f>
-        <x:v>6003.072</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$44,'Kosztorys siłowni'!$A$2:$A$44,A17)</x:f>
+        <x:v>6963.06</x:v>
       </x:c>
       <x:c r="E17" s="15" t="n">
         <x:f>D17/$B$7</x:f>
-        <x:v>0.025859012924854232</x:v>
+        <x:v>0.029172523535525553</x:v>
       </x:c>
       <x:c r="F17" s="6" t="str"/>
     </x:row>
@@ -552,16 +552,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C18" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A18)</x:f>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$44,'Kosztorys siłowni'!$A$2:$A$44,A18)</x:f>
         <x:v>8241.58</x:v>
       </x:c>
       <x:c r="D18" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A18)</x:f>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$44,'Kosztorys siłowni'!$A$2:$A$44,A18)</x:f>
         <x:v>9889.895999999999</x:v>
       </x:c>
       <x:c r="E18" s="15" t="n">
         <x:f>D18/$B$7</x:f>
-        <x:v>0.04260201251783489</x:v>
+        <x:v>0.041434832361619746</x:v>
       </x:c>
       <x:c r="F18" s="6" t="str"/>
     </x:row>
@@ -573,16 +573,16 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C19" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A19)</x:f>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$44,'Kosztorys siłowni'!$A$2:$A$44,A19)</x:f>
         <x:v>27625.239999999998</x:v>
       </x:c>
       <x:c r="D19" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A19)</x:f>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$44,'Kosztorys siłowni'!$A$2:$A$44,A19)</x:f>
         <x:v>33150.288</x:v>
       </x:c>
       <x:c r="E19" s="15" t="n">
         <x:f>D19/$B$7</x:f>
-        <x:v>0.14279917446511387</x:v>
+        <x:v>0.13888686251295412</x:v>
       </x:c>
       <x:c r="F19" s="6" t="str"/>
     </x:row>
@@ -591,63 +591,84 @@
         <x:v>Drabinki i drobny sprzęt</x:v>
       </x:c>
       <x:c r="B20" s="6" t="n">
-        <x:v>4</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C20" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A20)</x:f>
-        <x:v>5722.41</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$44,'Kosztorys siłowni'!$A$2:$A$44,A20)</x:f>
+        <x:v>6410.709999999999</x:v>
       </x:c>
       <x:c r="D20" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A20)</x:f>
-        <x:v>6866.892</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$44,'Kosztorys siłowni'!$A$2:$A$44,A20)</x:f>
+        <x:v>7692.852</x:v>
       </x:c>
       <x:c r="E20" s="15" t="n">
         <x:f>D20/$B$7</x:f>
-        <x:v>0.02958002985497727</x:v>
+        <x:v>0.03223006925479815</x:v>
       </x:c>
       <x:c r="F20" s="6" t="str"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="6" t="str">
-        <x:v>Opcjonalne uzupełnienie</x:v>
+        <x:v>Trening funkcjonalny</x:v>
       </x:c>
       <x:c r="B21" s="6" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C21" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A21)</x:f>
-        <x:v>3825.89</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$44,'Kosztorys siłowni'!$A$2:$A$44,A21)</x:f>
+        <x:v>3961.1600000000003</x:v>
       </x:c>
       <x:c r="D21" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A21)</x:f>
-        <x:v>4591.067999999999</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$44,'Kosztorys siłowni'!$A$2:$A$44,A21)</x:f>
+        <x:v>4753.392000000001</x:v>
       </x:c>
       <x:c r="E21" s="15" t="n">
         <x:f>D21/$B$7</x:f>
-        <x:v>0.019776622161267538</x:v>
+        <x:v>0.019914870759921485</x:v>
       </x:c>
       <x:c r="F21" s="6" t="str"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="6" t="str">
-        <x:v>Wyposażenie AV</x:v>
+        <x:v>Opcjonalne uzupełnienie</x:v>
       </x:c>
       <x:c r="B22" s="6" t="n">
-        <x:v>8</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C22" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$35,'Kosztorys siłowni'!$A$2:$A$35,A22)</x:f>
-        <x:v>17762.98</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$44,'Kosztorys siłowni'!$A$2:$A$44,A22)</x:f>
+        <x:v>3825.89</x:v>
       </x:c>
       <x:c r="D22" s="10" t="n">
-        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$35,'Kosztorys siłowni'!$A$2:$A$35,A22)</x:f>
-        <x:v>21315.575999999997</x:v>
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$44,'Kosztorys siłowni'!$A$2:$A$44,A22)</x:f>
+        <x:v>4591.067999999999</x:v>
       </x:c>
       <x:c r="E22" s="15" t="n">
         <x:f>D22/$B$7</x:f>
-        <x:v>0.09181961423829542</x:v>
+        <x:v>0.01923479609298185</x:v>
       </x:c>
       <x:c r="F22" s="6" t="str"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="6" t="str">
+        <x:v>Wyposażenie AV</x:v>
+      </x:c>
+      <x:c r="B23" s="6" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C23" s="10" t="n">
+        <x:f>SUMIFS('Kosztorys siłowni'!$F$2:$F$44,'Kosztorys siłowni'!$A$2:$A$44,A23)</x:f>
+        <x:v>17762.98</x:v>
+      </x:c>
+      <x:c r="D23" s="10" t="n">
+        <x:f>SUMIFS('Kosztorys siłowni'!$G$2:$G$44,'Kosztorys siłowni'!$A$2:$A$44,A23)</x:f>
+        <x:v>21315.575999999997</x:v>
+      </x:c>
+      <x:c r="E23" s="15" t="n">
+        <x:f>D23/$B$7</x:f>
+        <x:v>0.08930400463780055</x:v>
+      </x:c>
+      <x:c r="F23" s="6" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1372,315 +1393,567 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="6" t="str">
-        <x:v>Opcjonalne uzupełnienie</x:v>
+        <x:v>Trening funkcjonalny</x:v>
       </x:c>
       <x:c r="B26" s="19" t="str">
-        <x:v>Kettlebell żeliwny PRO, zestaw PROUD</x:v>
+        <x:v>Worek treningowy Powerbag PROUD, zestaw 5-25 kg</x:v>
       </x:c>
       <x:c r="C26" s="6" t="str">
         <x:v>1 zestaw</x:v>
       </x:c>
       <x:c r="D26" s="10" t="n">
-        <x:v>2625.99</x:v>
+        <x:v>1689.72</x:v>
       </x:c>
       <x:c r="E26" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F26" s="10" t="n">
         <x:f>D26</x:f>
-        <x:v>2625.99</x:v>
+        <x:v>1689.72</x:v>
       </x:c>
       <x:c r="G26" s="10" t="n">
         <x:f>F26*(1+E26)</x:f>
-        <x:v>3151.1879999999996</x:v>
+        <x:v>2027.664</x:v>
       </x:c>
       <x:c r="H26" s="19" t="str">
-        <x:v>https://trainingshowroom.com/hantle-i-kettlebells/3465-hantla-proud-kettlebell-zestaw.html</x:v>
+        <x:v>https://trainingshowroom.com/pilki-i-worki/2609-worek-treningowy-powerbag-proud.html</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="6" t="str">
-        <x:v>Opcjonalne uzupełnienie</x:v>
+        <x:v>Trening funkcjonalny</x:v>
       </x:c>
       <x:c r="B27" s="19" t="str">
-        <x:v>Podłoga gumowa Standard PROUD 15 mm pod kettlebell</x:v>
+        <x:v>Stojak na worki treningowe Powerbag PROUD</x:v>
       </x:c>
       <x:c r="C27" s="6" t="str">
-        <x:v>10 szt.</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D27" s="10" t="n">
-        <x:v>1199.9</x:v>
+        <x:v>2101.8</x:v>
       </x:c>
       <x:c r="E27" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F27" s="10" t="n">
         <x:f>D27</x:f>
-        <x:v>1199.9</x:v>
+        <x:v>2101.8</x:v>
       </x:c>
       <x:c r="G27" s="10" t="n">
         <x:f>F27*(1+E27)</x:f>
-        <x:v>1439.88</x:v>
+        <x:v>2522.1600000000003</x:v>
       </x:c>
       <x:c r="H27" s="19" t="str">
-        <x:v>https://trainingshowroom.com/podlogi/3427-podloga-gumowa-standard-proud.html</x:v>
+        <x:v>https://trainingshowroom.com/pilki-i-worki/2609-worek-treningowy-powerbag-proud.html</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="6" t="str">
-        <x:v>Wyposażenie AV</x:v>
+        <x:v>Ławki i gryfy</x:v>
       </x:c>
       <x:c r="B28" s="19" t="str">
-        <x:v>Lustra na jedną ścianę pomieszczenia</x:v>
+        <x:v>Sztanga specjalistyczna do martwego ciągu Hex Bar PROUD</x:v>
       </x:c>
       <x:c r="C28" s="6" t="str">
-        <x:v>ok. 16 m²</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D28" s="10" t="n">
-        <x:v>6500</x:v>
+        <x:v>799.99</x:v>
       </x:c>
       <x:c r="E28" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F28" s="10" t="n">
         <x:f>D28</x:f>
-        <x:v>6500</x:v>
+        <x:v>799.99</x:v>
       </x:c>
       <x:c r="G28" s="10" t="n">
         <x:f>F28*(1+E28)</x:f>
-        <x:v>7800</x:v>
+        <x:v>959.9879999999999</x:v>
       </x:c>
       <x:c r="H28" s="19" t="str">
-        <x:v>Cena orientacyjna, jedna pełna ściana</x:v>
+        <x:v>https://trainingshowroom.com/sztangi/2593-sztanga-specjalistyczna-do-martwego-ciagu-hex-bar.html</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="6" t="str">
-        <x:v>Wyposażenie AV</x:v>
+        <x:v>Trening funkcjonalny</x:v>
       </x:c>
       <x:c r="B29" s="19" t="str">
-        <x:v>Projektor Full HD Epson EB-FH52</x:v>
+        <x:v>Skakanka treningowa Speed Rope 2.0 PROUD</x:v>
       </x:c>
       <x:c r="C29" s="6" t="str">
-        <x:v>1</x:v>
+        <x:v>4 szt.</x:v>
       </x:c>
       <x:c r="D29" s="10" t="n">
-        <x:v>4559</x:v>
+        <x:v>169.64</x:v>
       </x:c>
       <x:c r="E29" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F29" s="10" t="n">
         <x:f>D29</x:f>
-        <x:v>4559</x:v>
+        <x:v>169.64</x:v>
       </x:c>
       <x:c r="G29" s="10" t="n">
         <x:f>F29*(1+E29)</x:f>
-        <x:v>5470.8</x:v>
+        <x:v>203.56799999999998</x:v>
       </x:c>
       <x:c r="H29" s="19" t="str">
-        <x:v>https://www.x-kom.pl/p/1224184-projektor-epson-eb-fh52.html</x:v>
+        <x:v>https://trainingshowroom.com/sprzet-fitness/2544-skakanka-treningowa-proud-speed-rope-20.html</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="6" t="str">
-        <x:v>Wyposażenie AV</x:v>
+        <x:v>Drabinki i drobny sprzęt</x:v>
       </x:c>
       <x:c r="B30" s="19" t="str">
-        <x:v>Ekran projekcyjny elektryczny Avtek Cinema Electric 300P</x:v>
+        <x:v>Pas kulturystyczny z łańcuchem PROUD</x:v>
       </x:c>
       <x:c r="C30" s="6" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D30" s="10" t="n">
-        <x:v>1419</x:v>
+        <x:v>105.03</x:v>
       </x:c>
       <x:c r="E30" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F30" s="10" t="n">
         <x:f>D30</x:f>
-        <x:v>1419</x:v>
+        <x:v>105.03</x:v>
       </x:c>
       <x:c r="G30" s="10" t="n">
         <x:f>F30*(1+E30)</x:f>
-        <x:v>1702.8</x:v>
+        <x:v>126.036</x:v>
       </x:c>
       <x:c r="H30" s="19" t="str">
-        <x:v>https://www.x-kom.pl/p/711610-ekran-projekcyjny-avtek-ekran-elektryczny-cinema-electric-300p.html</x:v>
+        <x:v>https://trainingshowroom.com/akcesoria/2545-pas-kulturystyczny-z-lancuchem-proud.html</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="6" t="str">
-        <x:v>Wyposażenie AV</x:v>
+        <x:v>Drabinki i drobny sprzęt</x:v>
       </x:c>
       <x:c r="B31" s="19" t="str">
-        <x:v>Kabel HDMI światłowodowy 20 m Claroc</x:v>
+        <x:v>Uchwyt obrotowy Land Mine PROUD EDGE</x:v>
       </x:c>
       <x:c r="C31" s="6" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D31" s="10" t="n">
-        <x:v>209</x:v>
+        <x:v>299</x:v>
       </x:c>
       <x:c r="E31" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F31" s="10" t="n">
         <x:f>D31</x:f>
-        <x:v>209</x:v>
+        <x:v>299</x:v>
       </x:c>
       <x:c r="G31" s="10" t="n">
         <x:f>F31*(1+E31)</x:f>
-        <x:v>250.79999999999998</x:v>
+        <x:v>358.8</x:v>
       </x:c>
       <x:c r="H31" s="19" t="str">
-        <x:v>https://www.x-kom.pl/p/1277224-kabel-hdmi-claroc-optyczny-hdmi-21-8k-120hz-20m.html</x:v>
+        <x:v>https://trainingshowroom.com/proud-edge/3552-uchwyt-obrotowy-land-mine-proud-edge.html</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="6" t="str">
-        <x:v>Wyposażenie AV</x:v>
+        <x:v>Drabinki i drobny sprzęt</x:v>
       </x:c>
       <x:c r="B32" s="19" t="str">
-        <x:v>Zestaw stereo Bluetooth Triangle AIO TWIN</x:v>
+        <x:v>Karabińczyk do wyciągu, zestaw PROUD</x:v>
       </x:c>
       <x:c r="C32" s="6" t="str">
-        <x:v>1 komplet</x:v>
+        <x:v>1 zestaw</x:v>
       </x:c>
       <x:c r="D32" s="10" t="n">
-        <x:v>2990</x:v>
+        <x:v>43.92</x:v>
       </x:c>
       <x:c r="E32" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F32" s="10" t="n">
         <x:f>D32</x:f>
-        <x:v>2990</x:v>
+        <x:v>43.92</x:v>
       </x:c>
       <x:c r="G32" s="10" t="n">
         <x:f>F32*(1+E32)</x:f>
-        <x:v>3588</x:v>
+        <x:v>52.704</x:v>
       </x:c>
       <x:c r="H32" s="19" t="str">
-        <x:v>https://avstore.pl/monitory-aktywne/triangle-aio-twin-aktywne-kolumny-podstawkowe-z-bluetooth-wi-fi.html</x:v>
+        <x:v>https://trainingshowroom.com/maszyny-silowe/3398-karabinczyk-do-wyciagu-zestaw-proud.html?search_query=Karabinczyk</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="6" t="str">
-        <x:v>Wyposażenie AV</x:v>
+        <x:v>Drabinki i drobny sprzęt</x:v>
       </x:c>
       <x:c r="B33" s="19" t="str">
-        <x:v>Zestaw mikrofonowy nagłowny Tonsil ZP 12</x:v>
+        <x:v>Uchwyt do wyciągu linowy PROUD</x:v>
       </x:c>
       <x:c r="C33" s="6" t="str">
-        <x:v>1 komplet</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D33" s="10" t="n">
-        <x:v>1699</x:v>
+        <x:v>74.73</x:v>
       </x:c>
       <x:c r="E33" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F33" s="10" t="n">
         <x:f>D33</x:f>
-        <x:v>1699</x:v>
+        <x:v>74.73</x:v>
       </x:c>
       <x:c r="G33" s="10" t="n">
         <x:f>F33*(1+E33)</x:f>
-        <x:v>2038.8</x:v>
+        <x:v>89.676</x:v>
       </x:c>
       <x:c r="H33" s="19" t="str">
-        <x:v>https://avstore.pl/naglosnienie-przenosne/zestaw-tonsil-zp-12-przenosny-bezprzewodowy-system-naglosnieniowy-pa-mikrofon-uhf-mikrofon-naglowny-statyw-m502-102.html</x:v>
+        <x:v>https://trainingshowroom.com/maszyny-silowe/2624-uchwyt-do-wyciagu-linowy-proud.html</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="6" t="str">
-        <x:v>Wyposażenie AV</x:v>
+        <x:v>Drabinki i drobny sprzęt</x:v>
       </x:c>
       <x:c r="B34" s="19" t="str">
-        <x:v>Uchwyty ścienne do głośników Gravity SP WMBS 30 B</x:v>
+        <x:v>Pojedynczy uchwyt do wyciągu obrotowy ogumowany PROUD</x:v>
       </x:c>
       <x:c r="C34" s="6" t="str">
         <x:v>2 szt.</x:v>
       </x:c>
       <x:c r="D34" s="10" t="n">
-        <x:v>319.98</x:v>
+        <x:v>165.62</x:v>
       </x:c>
       <x:c r="E34" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F34" s="10" t="n">
         <x:f>D34</x:f>
-        <x:v>319.98</x:v>
+        <x:v>165.62</x:v>
       </x:c>
       <x:c r="G34" s="10" t="n">
         <x:f>F34*(1+E34)</x:f>
-        <x:v>383.976</x:v>
+        <x:v>198.744</x:v>
       </x:c>
       <x:c r="H34" s="19" t="str">
-        <x:v>https://www.ablosklep.com/gravity-sp-wmbs-30-b-wychylny-obrotowy-uchwyt-scienny-do-glosnikow-do-30-kg-czarny-p-3991.html</x:v>
+        <x:v>https://trainingshowroom.com/maszyny-silowe/2587-pojedynczy-uchwyt-do-wyciagu-obrotowy-ogumowany-proud.html</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="6" t="str">
-        <x:v>Wyposażenie AV</x:v>
+        <x:v>Opcjonalne uzupełnienie</x:v>
       </x:c>
       <x:c r="B35" s="19" t="str">
-        <x:v>Kabel audio mini jack 3,5 mm - 2x RCA 10 m Lindy</x:v>
+        <x:v>Kettlebell żeliwny PRO, zestaw PROUD</x:v>
       </x:c>
       <x:c r="C35" s="6" t="str">
-        <x:v>1</x:v>
+        <x:v>1 zestaw</x:v>
       </x:c>
       <x:c r="D35" s="10" t="n">
-        <x:v>67</x:v>
+        <x:v>2625.99</x:v>
       </x:c>
       <x:c r="E35" s="7" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="F35" s="10" t="n">
         <x:f>D35</x:f>
-        <x:v>67</x:v>
+        <x:v>2625.99</x:v>
       </x:c>
       <x:c r="G35" s="10" t="n">
         <x:f>F35*(1+E35)</x:f>
+        <x:v>3151.1879999999996</x:v>
+      </x:c>
+      <x:c r="H35" s="19" t="str">
+        <x:v>https://trainingshowroom.com/hantle-i-kettlebells/3465-hantla-proud-kettlebell-zestaw.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="6" t="str">
+        <x:v>Opcjonalne uzupełnienie</x:v>
+      </x:c>
+      <x:c r="B36" s="19" t="str">
+        <x:v>Podłoga gumowa Standard PROUD 15 mm pod kettlebell</x:v>
+      </x:c>
+      <x:c r="C36" s="6" t="str">
+        <x:v>10 szt.</x:v>
+      </x:c>
+      <x:c r="D36" s="10" t="n">
+        <x:v>1199.9</x:v>
+      </x:c>
+      <x:c r="E36" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F36" s="10" t="n">
+        <x:f>D36</x:f>
+        <x:v>1199.9</x:v>
+      </x:c>
+      <x:c r="G36" s="10" t="n">
+        <x:f>F36*(1+E36)</x:f>
+        <x:v>1439.88</x:v>
+      </x:c>
+      <x:c r="H36" s="19" t="str">
+        <x:v>https://trainingshowroom.com/podlogi/3427-podloga-gumowa-standard-proud.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="6" t="str">
+        <x:v>Wyposażenie AV</x:v>
+      </x:c>
+      <x:c r="B37" s="19" t="str">
+        <x:v>Lustra na jedną ścianę pomieszczenia</x:v>
+      </x:c>
+      <x:c r="C37" s="6" t="str">
+        <x:v>ok. 16 m²</x:v>
+      </x:c>
+      <x:c r="D37" s="10" t="n">
+        <x:v>6500</x:v>
+      </x:c>
+      <x:c r="E37" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F37" s="10" t="n">
+        <x:f>D37</x:f>
+        <x:v>6500</x:v>
+      </x:c>
+      <x:c r="G37" s="10" t="n">
+        <x:f>F37*(1+E37)</x:f>
+        <x:v>7800</x:v>
+      </x:c>
+      <x:c r="H37" s="19" t="str">
+        <x:v>Cena orientacyjna, jedna pełna ściana</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="6" t="str">
+        <x:v>Wyposażenie AV</x:v>
+      </x:c>
+      <x:c r="B38" s="19" t="str">
+        <x:v>Projektor Full HD Epson EB-FH52</x:v>
+      </x:c>
+      <x:c r="C38" s="6" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D38" s="10" t="n">
+        <x:v>4559</x:v>
+      </x:c>
+      <x:c r="E38" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F38" s="10" t="n">
+        <x:f>D38</x:f>
+        <x:v>4559</x:v>
+      </x:c>
+      <x:c r="G38" s="10" t="n">
+        <x:f>F38*(1+E38)</x:f>
+        <x:v>5470.8</x:v>
+      </x:c>
+      <x:c r="H38" s="19" t="str">
+        <x:v>https://www.x-kom.pl/p/1224184-projektor-epson-eb-fh52.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="6" t="str">
+        <x:v>Wyposażenie AV</x:v>
+      </x:c>
+      <x:c r="B39" s="19" t="str">
+        <x:v>Ekran projekcyjny elektryczny Avtek Cinema Electric 300P</x:v>
+      </x:c>
+      <x:c r="C39" s="6" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D39" s="10" t="n">
+        <x:v>1419</x:v>
+      </x:c>
+      <x:c r="E39" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F39" s="10" t="n">
+        <x:f>D39</x:f>
+        <x:v>1419</x:v>
+      </x:c>
+      <x:c r="G39" s="10" t="n">
+        <x:f>F39*(1+E39)</x:f>
+        <x:v>1702.8</x:v>
+      </x:c>
+      <x:c r="H39" s="19" t="str">
+        <x:v>https://www.x-kom.pl/p/711610-ekran-projekcyjny-avtek-ekran-elektryczny-cinema-electric-300p.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="6" t="str">
+        <x:v>Wyposażenie AV</x:v>
+      </x:c>
+      <x:c r="B40" s="19" t="str">
+        <x:v>Kabel HDMI światłowodowy 20 m Claroc</x:v>
+      </x:c>
+      <x:c r="C40" s="6" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D40" s="10" t="n">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="E40" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F40" s="10" t="n">
+        <x:f>D40</x:f>
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="G40" s="10" t="n">
+        <x:f>F40*(1+E40)</x:f>
+        <x:v>250.79999999999998</x:v>
+      </x:c>
+      <x:c r="H40" s="19" t="str">
+        <x:v>https://www.x-kom.pl/p/1277224-kabel-hdmi-claroc-optyczny-hdmi-21-8k-120hz-20m.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="6" t="str">
+        <x:v>Wyposażenie AV</x:v>
+      </x:c>
+      <x:c r="B41" s="19" t="str">
+        <x:v>Zestaw stereo Bluetooth Triangle AIO TWIN</x:v>
+      </x:c>
+      <x:c r="C41" s="6" t="str">
+        <x:v>1 komplet</x:v>
+      </x:c>
+      <x:c r="D41" s="10" t="n">
+        <x:v>2990</x:v>
+      </x:c>
+      <x:c r="E41" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F41" s="10" t="n">
+        <x:f>D41</x:f>
+        <x:v>2990</x:v>
+      </x:c>
+      <x:c r="G41" s="10" t="n">
+        <x:f>F41*(1+E41)</x:f>
+        <x:v>3588</x:v>
+      </x:c>
+      <x:c r="H41" s="19" t="str">
+        <x:v>https://avstore.pl/monitory-aktywne/triangle-aio-twin-aktywne-kolumny-podstawkowe-z-bluetooth-wi-fi.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="6" t="str">
+        <x:v>Wyposażenie AV</x:v>
+      </x:c>
+      <x:c r="B42" s="19" t="str">
+        <x:v>Zestaw mikrofonowy nagłowny Tonsil ZP 12</x:v>
+      </x:c>
+      <x:c r="C42" s="6" t="str">
+        <x:v>1 komplet</x:v>
+      </x:c>
+      <x:c r="D42" s="10" t="n">
+        <x:v>1699</x:v>
+      </x:c>
+      <x:c r="E42" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F42" s="10" t="n">
+        <x:f>D42</x:f>
+        <x:v>1699</x:v>
+      </x:c>
+      <x:c r="G42" s="10" t="n">
+        <x:f>F42*(1+E42)</x:f>
+        <x:v>2038.8</x:v>
+      </x:c>
+      <x:c r="H42" s="19" t="str">
+        <x:v>https://avstore.pl/naglosnienie-przenosne/zestaw-tonsil-zp-12-przenosny-bezprzewodowy-system-naglosnieniowy-pa-mikrofon-uhf-mikrofon-naglowny-statyw-m502-102.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="6" t="str">
+        <x:v>Wyposażenie AV</x:v>
+      </x:c>
+      <x:c r="B43" s="19" t="str">
+        <x:v>Uchwyty ścienne do głośników Gravity SP WMBS 30 B</x:v>
+      </x:c>
+      <x:c r="C43" s="6" t="str">
+        <x:v>2 szt.</x:v>
+      </x:c>
+      <x:c r="D43" s="10" t="n">
+        <x:v>319.98</x:v>
+      </x:c>
+      <x:c r="E43" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F43" s="10" t="n">
+        <x:f>D43</x:f>
+        <x:v>319.98</x:v>
+      </x:c>
+      <x:c r="G43" s="10" t="n">
+        <x:f>F43*(1+E43)</x:f>
+        <x:v>383.976</x:v>
+      </x:c>
+      <x:c r="H43" s="19" t="str">
+        <x:v>https://www.ablosklep.com/gravity-sp-wmbs-30-b-wychylny-obrotowy-uchwyt-scienny-do-glosnikow-do-30-kg-czarny-p-3991.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="6" t="str">
+        <x:v>Wyposażenie AV</x:v>
+      </x:c>
+      <x:c r="B44" s="19" t="str">
+        <x:v>Kabel audio mini jack 3,5 mm - 2x RCA 10 m Lindy</x:v>
+      </x:c>
+      <x:c r="C44" s="6" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D44" s="10" t="n">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="E44" s="7" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F44" s="10" t="n">
+        <x:f>D44</x:f>
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="G44" s="10" t="n">
+        <x:f>F44*(1+E44)</x:f>
         <x:v>80.39999999999999</x:v>
       </x:c>
-      <x:c r="H35" s="19" t="str">
+      <x:c r="H44" s="19" t="str">
         <x:v>https://sklep.rms.pl/lindy-35337-kabel-mini-jack-3-5mm-2x-rca-cromo-line-10m</x:v>
       </x:c>
     </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="6"/>
-      <x:c r="B36" s="6"/>
-      <x:c r="C36" s="6"/>
-      <x:c r="D36" s="10"/>
-      <x:c r="E36" s="6"/>
-      <x:c r="F36" s="10"/>
-      <x:c r="G36" s="10"/>
-      <x:c r="H36" s="6"/>
-    </x:row>
-    <x:row r="37">
-      <x:c r="A37" s="17" t="str">
+    <x:row r="45">
+      <x:c r="A45" s="6"/>
+      <x:c r="B45" s="6"/>
+      <x:c r="C45" s="6"/>
+      <x:c r="D45" s="10"/>
+      <x:c r="E45" s="6"/>
+      <x:c r="F45" s="10"/>
+      <x:c r="G45" s="10"/>
+      <x:c r="H45" s="6"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="17" t="str">
         <x:v>Razem</x:v>
       </x:c>
-      <x:c r="B37" s="17"/>
-      <x:c r="C37" s="17"/>
-      <x:c r="D37" s="18"/>
-      <x:c r="E37" s="17"/>
-      <x:c r="F37" s="18" t="n">
-        <x:f>SUM(F2:F35)</x:f>
-        <x:v>193455.18</x:v>
-      </x:c>
-      <x:c r="G37" s="18" t="n">
-        <x:f>SUM(G2:G35)</x:f>
-        <x:v>232146.21599999993</x:v>
-      </x:c>
-      <x:c r="H37" s="17"/>
+      <x:c r="B46" s="17"/>
+      <x:c r="C46" s="17"/>
+      <x:c r="D46" s="18"/>
+      <x:c r="E46" s="17"/>
+      <x:c r="F46" s="18" t="n">
+        <x:f>SUM(F2:F44)</x:f>
+        <x:v>198904.63</x:v>
+      </x:c>
+      <x:c r="G46" s="18" t="n">
+        <x:f>SUM(G2:G44)</x:f>
+        <x:v>238685.55599999992</x:v>
+      </x:c>
+      <x:c r="H46" s="17"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A37:C37"/>
+    <x:mergeCell ref="A46:C46"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>